<commit_message>
update M7 compare sheet
</commit_message>
<xml_diff>
--- a/CDAtoFHIRExamples/Input/USCDI_v3_Myra_compare.xlsx
+++ b/CDAtoFHIRExamples/Input/USCDI_v3_Myra_compare.xlsx
@@ -8,20 +8,37 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repos\CCDAtoFHIRSamples\CDAtoFHIRExamples\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{1F92A17B-8E6A-4697-86B4-18567479EC8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6552BFC3-6157-4B2D-8C5D-EF0B87D11EAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{AD9AA5AD-85CE-4E99-8021-1D0325A3266B}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{AD9AA5AD-85CE-4E99-8021-1D0325A3266B}"/>
   </bookViews>
   <sheets>
     <sheet name="USCDI_v3_Myra_v6" sheetId="1" r:id="rId1"/>
     <sheet name="USCDI_v3_Myra_v7" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames>
+    <definedName name="name6">USCDI_v3_Myra_v6!$C:$C</definedName>
+    <definedName name="name6a">USCDI_v3_Myra_v6!$C:$D</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="851" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="249">
   <si>
     <t>USCDI Data Class</t>
   </si>
@@ -765,6 +782,9 @@
   </si>
   <si>
     <t>Omit</t>
+  </si>
+  <si>
+    <t>Found in Myra6</t>
   </si>
 </sst>
 </file>
@@ -907,7 +927,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1087,6 +1107,12 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -1248,9 +1274,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1629,7 +1657,7 @@
   <dimension ref="A1:G97"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="29" hidden="1" customWidth="1"/>
+    <col min="1" max="2" width="29" customWidth="1"/>
     <col min="3" max="3" width="58.54296875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="23.08984375" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
@@ -1669,8 +1697,8 @@
         <v>7</v>
       </c>
       <c r="C2" t="str">
-        <f>B2&amp;" - "&amp;B2</f>
-        <v>Substance (Reactant) - Substance (Reactant)</v>
+        <f>A2&amp;" - "&amp;B2</f>
+        <v>Allergies and Intolerances - Substance (Reactant)</v>
       </c>
       <c r="D2" t="s">
         <v>8</v>
@@ -1693,8 +1721,8 @@
         <v>11</v>
       </c>
       <c r="C3" t="str">
-        <f t="shared" ref="C3:C66" si="0">B3&amp;" - "&amp;B3</f>
-        <v>Reaction - Reaction</v>
+        <f t="shared" ref="C3:C66" si="0">A3&amp;" - "&amp;B3</f>
+        <v>Allergies and Intolerances - Reaction</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
@@ -1742,7 +1770,7 @@
       </c>
       <c r="C5" t="str">
         <f t="shared" si="0"/>
-        <v>SDOH Assessment - SDOH Assessment</v>
+        <v>Assessment and Plan of Treatment - SDOH Assessment</v>
       </c>
       <c r="D5" t="s">
         <v>8</v>
@@ -1766,7 +1794,7 @@
       </c>
       <c r="C6" t="str">
         <f t="shared" si="0"/>
-        <v>Care Team Member Name - Care Team Member Name</v>
+        <v>Care Team Member(s) - Care Team Member Name</v>
       </c>
       <c r="D6" t="s">
         <v>243</v>
@@ -1781,7 +1809,7 @@
       </c>
       <c r="C7" t="str">
         <f t="shared" si="0"/>
-        <v>Care Team Member Identifier - Care Team Member Identifier</v>
+        <v>Care Team Member(s) - Care Team Member Identifier</v>
       </c>
       <c r="D7" t="s">
         <v>243</v>
@@ -1796,7 +1824,7 @@
       </c>
       <c r="C8" t="str">
         <f t="shared" si="0"/>
-        <v>Care Team Member Location - Care Team Member Location</v>
+        <v>Care Team Member(s) - Care Team Member Location</v>
       </c>
       <c r="D8" t="s">
         <v>243</v>
@@ -1811,7 +1839,7 @@
       </c>
       <c r="C9" t="str">
         <f t="shared" si="0"/>
-        <v>Care Team Member Telecom - Care Team Member Telecom</v>
+        <v>Care Team Member(s) - Care Team Member Telecom</v>
       </c>
       <c r="D9" t="s">
         <v>243</v>
@@ -1826,7 +1854,7 @@
       </c>
       <c r="C10" t="str">
         <f t="shared" si="0"/>
-        <v>Care Team Member Role - Care Team Member Role</v>
+        <v>Care Team Member(s) - Care Team Member Role</v>
       </c>
       <c r="D10" t="s">
         <v>243</v>
@@ -1841,7 +1869,7 @@
       </c>
       <c r="C11" t="str">
         <f t="shared" si="0"/>
-        <v>Consultation Note - Consultation Note</v>
+        <v>Clinical Notes - Consultation Note</v>
       </c>
       <c r="D11" t="s">
         <v>8</v>
@@ -1865,7 +1893,7 @@
       </c>
       <c r="C12" t="str">
         <f t="shared" si="0"/>
-        <v>Discharge Summary Note - Discharge Summary Note</v>
+        <v>Clinical Notes - Discharge Summary Note</v>
       </c>
       <c r="D12" t="s">
         <v>245</v>
@@ -1880,7 +1908,7 @@
       </c>
       <c r="C13" t="str">
         <f t="shared" si="0"/>
-        <v>History &amp; Physical - History &amp; Physical</v>
+        <v>Clinical Notes - History &amp; Physical</v>
       </c>
       <c r="D13" t="s">
         <v>245</v>
@@ -1895,7 +1923,7 @@
       </c>
       <c r="C14" t="str">
         <f t="shared" si="0"/>
-        <v>Imaging Narrative - Imaging Narrative</v>
+        <v>Clinical Notes - Imaging Narrative</v>
       </c>
       <c r="D14" t="s">
         <v>245</v>
@@ -1910,7 +1938,7 @@
       </c>
       <c r="C15" t="str">
         <f t="shared" si="0"/>
-        <v>Laboratory Report Narrative - Laboratory Report Narrative</v>
+        <v>Clinical Notes - Laboratory Report Narrative</v>
       </c>
       <c r="D15" t="s">
         <v>245</v>
@@ -1925,7 +1953,7 @@
       </c>
       <c r="C16" t="str">
         <f t="shared" si="0"/>
-        <v>Pathology Report Narrative - Pathology Report Narrative</v>
+        <v>Clinical Notes - Pathology Report Narrative</v>
       </c>
       <c r="D16" t="s">
         <v>245</v>
@@ -1940,7 +1968,7 @@
       </c>
       <c r="C17" t="str">
         <f t="shared" si="0"/>
-        <v>Procedure Note - Procedure Note</v>
+        <v>Clinical Notes - Procedure Note</v>
       </c>
       <c r="D17" t="s">
         <v>245</v>
@@ -1955,7 +1983,7 @@
       </c>
       <c r="C18" t="str">
         <f t="shared" si="0"/>
-        <v>Progress Note - Progress Note</v>
+        <v>Clinical Notes - Progress Note</v>
       </c>
       <c r="D18" t="s">
         <v>245</v>
@@ -1970,7 +1998,7 @@
       </c>
       <c r="C19" t="str">
         <f t="shared" si="0"/>
-        <v>Encounter Diagnosis - Encounter Diagnosis</v>
+        <v>Encounter Information - Encounter Diagnosis</v>
       </c>
       <c r="D19" t="s">
         <v>8</v>
@@ -1994,7 +2022,7 @@
       </c>
       <c r="C20" t="str">
         <f t="shared" si="0"/>
-        <v>Encounter Disposition - Encounter Disposition</v>
+        <v>Encounter Information - Encounter Disposition</v>
       </c>
       <c r="D20" t="s">
         <v>243</v>
@@ -2009,7 +2037,7 @@
       </c>
       <c r="C21" t="str">
         <f t="shared" si="0"/>
-        <v>Encounter Location - Encounter Location</v>
+        <v>Encounter Information - Encounter Location</v>
       </c>
       <c r="D21" t="s">
         <v>243</v>
@@ -2024,7 +2052,7 @@
       </c>
       <c r="C22" t="str">
         <f t="shared" si="0"/>
-        <v>Encounter Time - Encounter Time</v>
+        <v>Encounter Information - Encounter Time</v>
       </c>
       <c r="D22" t="s">
         <v>8</v>
@@ -2048,7 +2076,7 @@
       </c>
       <c r="C23" t="str">
         <f t="shared" si="0"/>
-        <v>Encounter Type - Encounter Type</v>
+        <v>Encounter Information - Encounter Type</v>
       </c>
       <c r="D23" t="s">
         <v>8</v>
@@ -2072,7 +2100,7 @@
       </c>
       <c r="C24" t="str">
         <f t="shared" si="0"/>
-        <v>Patient Goals - Patient Goals</v>
+        <v>Goals - Patient Goals</v>
       </c>
       <c r="D24" t="s">
         <v>8</v>
@@ -2096,7 +2124,7 @@
       </c>
       <c r="C25" t="str">
         <f t="shared" si="0"/>
-        <v>SDOH Goals - SDOH Goals</v>
+        <v>Goals - SDOH Goals</v>
       </c>
       <c r="D25" t="s">
         <v>243</v>
@@ -2126,7 +2154,7 @@
       </c>
       <c r="C27" t="str">
         <f t="shared" si="0"/>
-        <v>SDOH Problems/Health Concerns - SDOH Problems/Health Concerns</v>
+        <v>Health Concerns - SDOH Problems/Health Concerns</v>
       </c>
       <c r="D27" t="s">
         <v>8</v>
@@ -2150,7 +2178,7 @@
       </c>
       <c r="C28" t="str">
         <f t="shared" si="0"/>
-        <v>Coverage Status - Coverage Status</v>
+        <v>Health Insurance Information - Coverage Status</v>
       </c>
       <c r="D28" t="s">
         <v>243</v>
@@ -2165,7 +2193,7 @@
       </c>
       <c r="C29" t="str">
         <f t="shared" si="0"/>
-        <v>Coverage Type - Coverage Type</v>
+        <v>Health Insurance Information - Coverage Type</v>
       </c>
       <c r="D29" t="s">
         <v>243</v>
@@ -2180,7 +2208,7 @@
       </c>
       <c r="C30" t="str">
         <f t="shared" si="0"/>
-        <v>Group Identifier - Group Identifier</v>
+        <v>Health Insurance Information - Group Identifier</v>
       </c>
       <c r="D30" t="s">
         <v>243</v>
@@ -2195,7 +2223,7 @@
       </c>
       <c r="C31" t="str">
         <f t="shared" si="0"/>
-        <v>Member Identifier - Member Identifier</v>
+        <v>Health Insurance Information - Member Identifier</v>
       </c>
       <c r="D31" t="s">
         <v>243</v>
@@ -2210,7 +2238,7 @@
       </c>
       <c r="C32" t="str">
         <f t="shared" si="0"/>
-        <v>Payer Identifier - Payer Identifier</v>
+        <v>Health Insurance Information - Payer Identifier</v>
       </c>
       <c r="D32" t="s">
         <v>243</v>
@@ -2225,7 +2253,7 @@
       </c>
       <c r="C33" t="str">
         <f t="shared" si="0"/>
-        <v>Relationship to Subscriber - Relationship to Subscriber</v>
+        <v>Health Insurance Information - Relationship to Subscriber</v>
       </c>
       <c r="D33" t="s">
         <v>243</v>
@@ -2240,7 +2268,7 @@
       </c>
       <c r="C34" t="str">
         <f t="shared" si="0"/>
-        <v>Subscriber Identifier - Subscriber Identifier</v>
+        <v>Health Insurance Information - Subscriber Identifier</v>
       </c>
       <c r="D34" t="s">
         <v>243</v>
@@ -2255,7 +2283,7 @@
       </c>
       <c r="C35" t="str">
         <f t="shared" si="0"/>
-        <v>Disability Status - Disability Status</v>
+        <v>Health Status/Assessments - Disability Status</v>
       </c>
       <c r="D35" t="s">
         <v>243</v>
@@ -2270,7 +2298,7 @@
       </c>
       <c r="C36" t="str">
         <f t="shared" si="0"/>
-        <v>Functional Status - Functional Status</v>
+        <v>Health Status/Assessments - Functional Status</v>
       </c>
       <c r="D36" t="s">
         <v>243</v>
@@ -2285,7 +2313,7 @@
       </c>
       <c r="C37" t="str">
         <f t="shared" si="0"/>
-        <v>Mental/Cognitive Status - Mental/Cognitive Status</v>
+        <v>Health Status/Assessments - Mental/Cognitive Status</v>
       </c>
       <c r="D37" t="s">
         <v>243</v>
@@ -2300,7 +2328,7 @@
       </c>
       <c r="C38" t="str">
         <f t="shared" si="0"/>
-        <v>Pregnancy Status - Pregnancy Status</v>
+        <v>Health Status/Assessments - Pregnancy Status</v>
       </c>
       <c r="D38" t="s">
         <v>241</v>
@@ -2339,7 +2367,7 @@
       </c>
       <c r="C40" t="str">
         <f t="shared" si="0"/>
-        <v>Tests - Tests</v>
+        <v>Laboratory - Tests</v>
       </c>
       <c r="D40" t="s">
         <v>8</v>
@@ -2363,7 +2391,7 @@
       </c>
       <c r="C41" t="str">
         <f t="shared" si="0"/>
-        <v>Values/Results - Values/Results</v>
+        <v>Laboratory - Values/Results</v>
       </c>
       <c r="D41" t="s">
         <v>8</v>
@@ -2387,7 +2415,7 @@
       </c>
       <c r="C42" t="str">
         <f t="shared" si="0"/>
-        <v>Result Interpretation - Result Interpretation</v>
+        <v>Laboratory - Result Interpretation</v>
       </c>
       <c r="D42" t="s">
         <v>241</v>
@@ -2402,7 +2430,7 @@
       </c>
       <c r="C43" t="str">
         <f t="shared" si="0"/>
-        <v>Result Reference Range - Result Reference Range</v>
+        <v>Laboratory - Result Reference Range</v>
       </c>
       <c r="D43" t="s">
         <v>8</v>
@@ -2426,7 +2454,7 @@
       </c>
       <c r="C44" t="str">
         <f t="shared" si="0"/>
-        <v>Result Status - Result Status</v>
+        <v>Laboratory - Result Status</v>
       </c>
       <c r="D44" t="s">
         <v>8</v>
@@ -2450,7 +2478,7 @@
       </c>
       <c r="C45" t="str">
         <f t="shared" si="0"/>
-        <v>Specimen Type - Specimen Type</v>
+        <v>Laboratory - Specimen Type</v>
       </c>
       <c r="D45" t="s">
         <v>241</v>
@@ -2489,7 +2517,7 @@
       </c>
       <c r="C47" t="str">
         <f t="shared" si="0"/>
-        <v>Dose - Dose</v>
+        <v>Medications - Dose</v>
       </c>
       <c r="D47" t="s">
         <v>8</v>
@@ -2513,7 +2541,7 @@
       </c>
       <c r="C48" t="str">
         <f t="shared" si="0"/>
-        <v>Dose Unit of Measure - Dose Unit of Measure</v>
+        <v>Medications - Dose Unit of Measure</v>
       </c>
       <c r="D48" t="s">
         <v>8</v>
@@ -2537,7 +2565,7 @@
       </c>
       <c r="C49" t="str">
         <f t="shared" si="0"/>
-        <v>Indication - Indication</v>
+        <v>Medications - Indication</v>
       </c>
       <c r="D49" t="s">
         <v>8</v>
@@ -2561,7 +2589,7 @@
       </c>
       <c r="C50" t="str">
         <f t="shared" si="0"/>
-        <v>Fill Status - Fill Status</v>
+        <v>Medications - Fill Status</v>
       </c>
       <c r="D50" t="s">
         <v>8</v>
@@ -2585,7 +2613,7 @@
       </c>
       <c r="C51" t="str">
         <f t="shared" si="0"/>
-        <v>Current Address - Current Address</v>
+        <v>Patient Demographics/Information - Current Address</v>
       </c>
       <c r="D51" t="s">
         <v>8</v>
@@ -2609,7 +2637,7 @@
       </c>
       <c r="C52" t="str">
         <f t="shared" si="0"/>
-        <v>Date of Birth - Date of Birth</v>
+        <v>Patient Demographics/Information - Date of Birth</v>
       </c>
       <c r="D52" t="s">
         <v>8</v>
@@ -2633,7 +2661,7 @@
       </c>
       <c r="C53" t="str">
         <f t="shared" si="0"/>
-        <v>Email Address - Email Address</v>
+        <v>Patient Demographics/Information - Email Address</v>
       </c>
       <c r="D53" t="s">
         <v>241</v>
@@ -2648,7 +2676,7 @@
       </c>
       <c r="C54" t="str">
         <f t="shared" si="0"/>
-        <v>Ethnicity - Ethnicity</v>
+        <v>Patient Demographics/Information - Ethnicity</v>
       </c>
       <c r="D54" t="s">
         <v>8</v>
@@ -2672,7 +2700,7 @@
       </c>
       <c r="C55" t="str">
         <f t="shared" si="0"/>
-        <v>First Name - First Name</v>
+        <v>Patient Demographics/Information - First Name</v>
       </c>
       <c r="D55" t="s">
         <v>8</v>
@@ -2696,7 +2724,7 @@
       </c>
       <c r="C56" t="str">
         <f t="shared" si="0"/>
-        <v>Gender Identity - Gender Identity</v>
+        <v>Patient Demographics/Information - Gender Identity</v>
       </c>
       <c r="D56" t="s">
         <v>247</v>
@@ -2711,7 +2739,7 @@
       </c>
       <c r="C57" t="str">
         <f t="shared" si="0"/>
-        <v>Last Name - Last Name</v>
+        <v>Patient Demographics/Information - Last Name</v>
       </c>
       <c r="D57" t="s">
         <v>8</v>
@@ -2735,7 +2763,7 @@
       </c>
       <c r="C58" t="str">
         <f t="shared" si="0"/>
-        <v>Phone Number - Phone Number</v>
+        <v>Patient Demographics/Information - Phone Number</v>
       </c>
       <c r="D58" t="s">
         <v>8</v>
@@ -2759,7 +2787,7 @@
       </c>
       <c r="C59" t="str">
         <f t="shared" si="0"/>
-        <v>Phone Number Type - Phone Number Type</v>
+        <v>Patient Demographics/Information - Phone Number Type</v>
       </c>
       <c r="D59" t="s">
         <v>8</v>
@@ -2783,7 +2811,7 @@
       </c>
       <c r="C60" t="str">
         <f t="shared" si="0"/>
-        <v>Preferred Language - Preferred Language</v>
+        <v>Patient Demographics/Information - Preferred Language</v>
       </c>
       <c r="D60" t="s">
         <v>8</v>
@@ -2807,7 +2835,7 @@
       </c>
       <c r="C61" t="str">
         <f t="shared" si="0"/>
-        <v>Previous Address - Previous Address</v>
+        <v>Patient Demographics/Information - Previous Address</v>
       </c>
       <c r="D61" t="s">
         <v>243</v>
@@ -2822,7 +2850,7 @@
       </c>
       <c r="C62" t="str">
         <f t="shared" si="0"/>
-        <v>Previous Name - Previous Name</v>
+        <v>Patient Demographics/Information - Previous Name</v>
       </c>
       <c r="D62" t="s">
         <v>243</v>
@@ -2837,7 +2865,7 @@
       </c>
       <c r="C63" t="str">
         <f t="shared" si="0"/>
-        <v>Race - Race</v>
+        <v>Patient Demographics/Information - Race</v>
       </c>
       <c r="D63" t="s">
         <v>8</v>
@@ -2861,7 +2889,7 @@
       </c>
       <c r="C64" t="str">
         <f t="shared" si="0"/>
-        <v>Related Person's Name - Related Person's Name</v>
+        <v>Patient Demographics/Information - Related Person's Name</v>
       </c>
       <c r="D64" t="s">
         <v>8</v>
@@ -2885,7 +2913,7 @@
       </c>
       <c r="C65" t="str">
         <f t="shared" si="0"/>
-        <v>Related Person's Relationship - Related Person's Relationship</v>
+        <v>Patient Demographics/Information - Related Person's Relationship</v>
       </c>
       <c r="D65" t="s">
         <v>8</v>
@@ -2909,7 +2937,7 @@
       </c>
       <c r="C66" t="str">
         <f t="shared" si="0"/>
-        <v>Sex - Sex</v>
+        <v>Patient Demographics/Information - Sex</v>
       </c>
       <c r="D66" t="s">
         <v>8</v>
@@ -2932,8 +2960,8 @@
         <v>135</v>
       </c>
       <c r="C67" t="str">
-        <f t="shared" ref="C67:C97" si="1">B67&amp;" - "&amp;B67</f>
-        <v>Sex Parameter for Clinical Use - Sex Parameter for Clinical Use</v>
+        <f t="shared" ref="C67:C97" si="1">A67&amp;" - "&amp;B67</f>
+        <v>Patient Demographics/Information - Sex Parameter for Clinical Use</v>
       </c>
       <c r="D67" t="s">
         <v>247</v>
@@ -2948,7 +2976,7 @@
       </c>
       <c r="C68" t="str">
         <f t="shared" si="1"/>
-        <v>Sexual Orientation - Sexual Orientation</v>
+        <v>Patient Demographics/Information - Sexual Orientation</v>
       </c>
       <c r="D68" t="s">
         <v>247</v>
@@ -2963,7 +2991,7 @@
       </c>
       <c r="C69" t="str">
         <f t="shared" si="1"/>
-        <v>Suffix - Suffix</v>
+        <v>Patient Demographics/Information - Suffix</v>
       </c>
       <c r="D69" t="s">
         <v>241</v>
@@ -2978,7 +3006,7 @@
       </c>
       <c r="C70" t="str">
         <f t="shared" si="1"/>
-        <v>Tribal Affiliation - Tribal Affiliation</v>
+        <v>Patient Demographics/Information - Tribal Affiliation</v>
       </c>
       <c r="D70" t="s">
         <v>243</v>
@@ -3017,7 +3045,7 @@
       </c>
       <c r="C72" t="str">
         <f t="shared" si="1"/>
-        <v>Date of Diagnosis - Date of Diagnosis</v>
+        <v>Problems - Date of Diagnosis</v>
       </c>
       <c r="D72" t="s">
         <v>8</v>
@@ -3041,7 +3069,7 @@
       </c>
       <c r="C73" t="str">
         <f t="shared" si="1"/>
-        <v>Date of Resolution - Date of Resolution</v>
+        <v>Problems - Date of Resolution</v>
       </c>
       <c r="D73" t="s">
         <v>8</v>
@@ -3089,7 +3117,7 @@
       </c>
       <c r="C75" t="str">
         <f t="shared" si="1"/>
-        <v>SDOH Interventions - SDOH Interventions</v>
+        <v>Procedures - SDOH Interventions</v>
       </c>
       <c r="D75" t="s">
         <v>8</v>
@@ -3113,7 +3141,7 @@
       </c>
       <c r="C76" t="str">
         <f t="shared" si="1"/>
-        <v>Performance Time - Performance Time</v>
+        <v>Procedures - Performance Time</v>
       </c>
       <c r="D76" t="s">
         <v>8</v>
@@ -3137,7 +3165,7 @@
       </c>
       <c r="C77" t="str">
         <f t="shared" si="1"/>
-        <v>Reason for Referral - Reason for Referral</v>
+        <v>Procedures - Reason for Referral</v>
       </c>
       <c r="D77" t="s">
         <v>243</v>
@@ -3152,7 +3180,7 @@
       </c>
       <c r="C78" t="str">
         <f t="shared" si="1"/>
-        <v>Author - Author</v>
+        <v>Provenance - Author</v>
       </c>
       <c r="D78" t="s">
         <v>8</v>
@@ -3176,7 +3204,7 @@
       </c>
       <c r="C79" t="str">
         <f t="shared" si="1"/>
-        <v>Author Organization - Author Organization</v>
+        <v>Provenance - Author Organization</v>
       </c>
       <c r="D79" t="s">
         <v>8</v>
@@ -3200,7 +3228,7 @@
       </c>
       <c r="C80" t="str">
         <f t="shared" si="1"/>
-        <v>Author Role - Author Role</v>
+        <v>Provenance - Author Role</v>
       </c>
       <c r="D80" t="s">
         <v>8</v>
@@ -3224,7 +3252,7 @@
       </c>
       <c r="C81" t="str">
         <f t="shared" si="1"/>
-        <v>Author Time Stamp - Author Time Stamp</v>
+        <v>Provenance - Author Time Stamp</v>
       </c>
       <c r="D81" t="s">
         <v>8</v>
@@ -3272,7 +3300,7 @@
       </c>
       <c r="C83" t="str">
         <f t="shared" si="1"/>
-        <v>Substance Use - Substance Use</v>
+        <v>Smoking Status - Substance Use</v>
       </c>
       <c r="D83" t="s">
         <v>242</v>
@@ -3287,7 +3315,7 @@
       </c>
       <c r="C84" t="str">
         <f t="shared" si="1"/>
-        <v>UDI - UDI</v>
+        <v>Unique Device Identifier(s) - UDI</v>
       </c>
       <c r="D84" t="s">
         <v>8</v>
@@ -3311,7 +3339,7 @@
       </c>
       <c r="C85" t="str">
         <f t="shared" si="1"/>
-        <v>BMI - BMI</v>
+        <v>Vital Signs - BMI</v>
       </c>
       <c r="D85" t="s">
         <v>241</v>
@@ -3326,7 +3354,7 @@
       </c>
       <c r="C86" t="str">
         <f t="shared" si="1"/>
-        <v>Blood Pressure (Diastolic) - Blood Pressure (Diastolic)</v>
+        <v>Vital Signs - Blood Pressure (Diastolic)</v>
       </c>
       <c r="D86" t="s">
         <v>241</v>
@@ -3341,7 +3369,7 @@
       </c>
       <c r="C87" t="str">
         <f t="shared" si="1"/>
-        <v>Blood Pressure (Systolic) - Blood Pressure (Systolic)</v>
+        <v>Vital Signs - Blood Pressure (Systolic)</v>
       </c>
       <c r="D87" t="s">
         <v>241</v>
@@ -3356,7 +3384,7 @@
       </c>
       <c r="C88" t="str">
         <f t="shared" si="1"/>
-        <v>Body Height - Body Height</v>
+        <v>Vital Signs - Body Height</v>
       </c>
       <c r="D88" t="s">
         <v>241</v>
@@ -3371,7 +3399,7 @@
       </c>
       <c r="C89" t="str">
         <f t="shared" si="1"/>
-        <v>Body Temperature - Body Temperature</v>
+        <v>Vital Signs - Body Temperature</v>
       </c>
       <c r="D89" t="s">
         <v>241</v>
@@ -3386,7 +3414,7 @@
       </c>
       <c r="C90" t="str">
         <f t="shared" si="1"/>
-        <v>Body Weight - Body Weight</v>
+        <v>Vital Signs - Body Weight</v>
       </c>
       <c r="D90" t="s">
         <v>241</v>
@@ -3401,7 +3429,7 @@
       </c>
       <c r="C91" t="str">
         <f t="shared" si="1"/>
-        <v>Heart Rate - Heart Rate</v>
+        <v>Vital Signs - Heart Rate</v>
       </c>
       <c r="D91" t="s">
         <v>241</v>
@@ -3425,7 +3453,7 @@
       </c>
       <c r="C92" t="str">
         <f t="shared" si="1"/>
-        <v>Inhaled Oxygen Concentration - Inhaled Oxygen Concentration</v>
+        <v>Vital Signs - Inhaled Oxygen Concentration</v>
       </c>
       <c r="D92" t="s">
         <v>241</v>
@@ -3440,7 +3468,7 @@
       </c>
       <c r="C93" t="str">
         <f t="shared" si="1"/>
-        <v>Pediatric BMI for Age - Pediatric BMI for Age</v>
+        <v>Vital Signs - Pediatric BMI for Age</v>
       </c>
       <c r="D93" t="s">
         <v>241</v>
@@ -3455,7 +3483,7 @@
       </c>
       <c r="C94" t="str">
         <f t="shared" si="1"/>
-        <v>Pediatric Head Circumference - Pediatric Head Circumference</v>
+        <v>Vital Signs - Pediatric Head Circumference</v>
       </c>
       <c r="D94" t="s">
         <v>241</v>
@@ -3470,7 +3498,7 @@
       </c>
       <c r="C95" t="str">
         <f t="shared" si="1"/>
-        <v>Pediatric Weight for Height - Pediatric Weight for Height</v>
+        <v>Vital Signs - Pediatric Weight for Height</v>
       </c>
       <c r="D95" t="s">
         <v>241</v>
@@ -3485,7 +3513,7 @@
       </c>
       <c r="C96" t="str">
         <f t="shared" si="1"/>
-        <v>Pulse Oximetry - Pulse Oximetry</v>
+        <v>Vital Signs - Pulse Oximetry</v>
       </c>
       <c r="D96" t="s">
         <v>241</v>
@@ -3500,7 +3528,7 @@
       </c>
       <c r="C97" t="str">
         <f t="shared" si="1"/>
-        <v>Respiratory Rate - Respiratory Rate</v>
+        <v>Vital Signs - Respiratory Rate</v>
       </c>
       <c r="D97" t="s">
         <v>241</v>
@@ -3513,1881 +3541,2269 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4C70803-C6D0-4941-8F3C-8CF7B7FD09A5}">
-  <dimension ref="A1:F97"/>
+  <dimension ref="A1:G97"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.90625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="59.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29" style="3" customWidth="1"/>
+    <col min="4" max="4" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="59.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
       <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2">
+      <c r="C2" s="3" t="str">
+        <f>VLOOKUP(A2&amp;" - "&amp;B2,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2">
         <v>782</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>9</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
       <c r="B3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3">
+      <c r="C3" s="3" t="str">
+        <f>VLOOKUP(A3&amp;" - "&amp;B3,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3">
         <v>802</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>12</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>14</v>
       </c>
       <c r="B4" t="s">
         <v>14</v>
       </c>
-      <c r="C4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4">
+      <c r="C4" s="3" t="str">
+        <f>VLOOKUP(A4&amp;" - "&amp;B4,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4">
         <v>1921</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>15</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>14</v>
       </c>
       <c r="B5" t="s">
         <v>17</v>
       </c>
-      <c r="C5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5">
+      <c r="C5" s="3" t="str">
+        <f>VLOOKUP(A5&amp;" - "&amp;B5,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5">
         <v>601</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>12</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>19</v>
       </c>
       <c r="B6" t="s">
         <v>20</v>
       </c>
-      <c r="C6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D6">
+      <c r="C6" s="3" t="str">
+        <f>VLOOKUP(A6&amp;" - "&amp;B6,name6a,2,FALSE)</f>
+        <v>To do</v>
+      </c>
+      <c r="D6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6">
         <v>2731</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>156</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>19</v>
       </c>
       <c r="B7" t="s">
         <v>21</v>
       </c>
-      <c r="C7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7">
+      <c r="C7" s="3" t="str">
+        <f>VLOOKUP(A7&amp;" - "&amp;B7,name6a,2,FALSE)</f>
+        <v>To do</v>
+      </c>
+      <c r="D7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7">
         <v>2754</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>239</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>19</v>
       </c>
       <c r="B8" t="s">
         <v>22</v>
       </c>
-      <c r="C8" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8">
+      <c r="C8" s="3" t="str">
+        <f>VLOOKUP(A8&amp;" - "&amp;B8,name6a,2,FALSE)</f>
+        <v>To do</v>
+      </c>
+      <c r="D8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8">
         <v>2757</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>98</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
       <c r="B9" t="s">
         <v>23</v>
       </c>
-      <c r="C9" t="s">
-        <v>8</v>
-      </c>
-      <c r="D9">
+      <c r="C9" s="3" t="str">
+        <f>VLOOKUP(A9&amp;" - "&amp;B9,name6a,2,FALSE)</f>
+        <v>To do</v>
+      </c>
+      <c r="D9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9">
         <v>2762</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>114</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>19</v>
       </c>
       <c r="B10" t="s">
         <v>24</v>
       </c>
-      <c r="C10" t="s">
-        <v>8</v>
-      </c>
-      <c r="D10">
+      <c r="C10" s="3" t="str">
+        <f>VLOOKUP(A10&amp;" - "&amp;B10,name6a,2,FALSE)</f>
+        <v>To do</v>
+      </c>
+      <c r="D10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10">
         <v>2755</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>45</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
       <c r="B11" t="s">
         <v>26</v>
       </c>
-      <c r="C11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D11">
+      <c r="C11" s="3" t="str">
+        <f>VLOOKUP(A11&amp;" - "&amp;B11,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D11" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11">
         <v>2522</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>27</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>25</v>
       </c>
       <c r="B12" t="s">
         <v>29</v>
       </c>
-      <c r="C12" t="s">
-        <v>8</v>
-      </c>
-      <c r="D12">
+      <c r="C12" s="3" t="str">
+        <f>VLOOKUP(A12&amp;" - "&amp;B12,name6a,2,FALSE)</f>
+        <v>Note - no need for example</v>
+      </c>
+      <c r="D12" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12">
         <v>2553</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
         <v>27</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>25</v>
       </c>
       <c r="B13" t="s">
         <v>30</v>
       </c>
-      <c r="C13" t="s">
-        <v>8</v>
-      </c>
-      <c r="D13">
+      <c r="C13" s="3" t="str">
+        <f>VLOOKUP(A13&amp;" - "&amp;B13,name6a,2,FALSE)</f>
+        <v>Note - no need for example</v>
+      </c>
+      <c r="D13" t="s">
+        <v>8</v>
+      </c>
+      <c r="E13">
         <v>2573</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>27</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>25</v>
       </c>
       <c r="B14" t="s">
         <v>31</v>
       </c>
-      <c r="C14" t="s">
-        <v>8</v>
-      </c>
-      <c r="D14">
+      <c r="C14" s="3" t="str">
+        <f>VLOOKUP(A14&amp;" - "&amp;B14,name6a,2,FALSE)</f>
+        <v>Note - no need for example</v>
+      </c>
+      <c r="D14" t="s">
+        <v>8</v>
+      </c>
+      <c r="E14">
         <v>2593</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F14" t="s">
         <v>27</v>
       </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>25</v>
       </c>
       <c r="B15" t="s">
         <v>32</v>
       </c>
-      <c r="C15" t="s">
-        <v>8</v>
-      </c>
-      <c r="D15">
+      <c r="C15" s="3" t="str">
+        <f>VLOOKUP(A15&amp;" - "&amp;B15,name6a,2,FALSE)</f>
+        <v>Note - no need for example</v>
+      </c>
+      <c r="D15" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15">
         <v>2613</v>
       </c>
-      <c r="E15" t="s">
+      <c r="F15" t="s">
         <v>27</v>
       </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>25</v>
       </c>
       <c r="B16" t="s">
         <v>33</v>
       </c>
-      <c r="C16" t="s">
-        <v>8</v>
-      </c>
-      <c r="D16">
+      <c r="C16" s="3" t="str">
+        <f>VLOOKUP(A16&amp;" - "&amp;B16,name6a,2,FALSE)</f>
+        <v>Note - no need for example</v>
+      </c>
+      <c r="D16" t="s">
+        <v>8</v>
+      </c>
+      <c r="E16">
         <v>2633</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
         <v>27</v>
       </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>25</v>
       </c>
       <c r="B17" t="s">
         <v>34</v>
       </c>
-      <c r="C17" t="s">
-        <v>8</v>
-      </c>
-      <c r="D17">
+      <c r="C17" s="3" t="str">
+        <f>VLOOKUP(A17&amp;" - "&amp;B17,name6a,2,FALSE)</f>
+        <v>Note - no need for example</v>
+      </c>
+      <c r="D17" t="s">
+        <v>8</v>
+      </c>
+      <c r="E17">
         <v>2653</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
         <v>27</v>
       </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>25</v>
       </c>
       <c r="B18" t="s">
         <v>35</v>
       </c>
-      <c r="C18" t="s">
-        <v>8</v>
-      </c>
-      <c r="D18">
+      <c r="C18" s="3" t="str">
+        <f>VLOOKUP(A18&amp;" - "&amp;B18,name6a,2,FALSE)</f>
+        <v>Note - no need for example</v>
+      </c>
+      <c r="D18" t="s">
+        <v>8</v>
+      </c>
+      <c r="E18">
         <v>2673</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
         <v>27</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>36</v>
       </c>
       <c r="B19" t="s">
         <v>37</v>
       </c>
-      <c r="C19" t="s">
-        <v>8</v>
-      </c>
-      <c r="D19">
+      <c r="C19" s="3" t="str">
+        <f>VLOOKUP(A19&amp;" - "&amp;B19,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D19" t="s">
+        <v>8</v>
+      </c>
+      <c r="E19">
         <v>2428</v>
       </c>
-      <c r="E19" t="s">
+      <c r="F19" t="s">
         <v>12</v>
       </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>36</v>
       </c>
       <c r="B20" t="s">
         <v>39</v>
       </c>
-      <c r="C20" t="s">
-        <v>8</v>
-      </c>
-      <c r="D20">
+      <c r="C20" s="3" t="str">
+        <f>VLOOKUP(A20&amp;" - "&amp;B20,name6a,2,FALSE)</f>
+        <v>To do</v>
+      </c>
+      <c r="D20" t="s">
+        <v>8</v>
+      </c>
+      <c r="E20">
         <v>2373</v>
       </c>
-      <c r="E20" t="s">
+      <c r="F20" t="s">
         <v>227</v>
       </c>
-      <c r="F20" t="s">
+      <c r="G20" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>36</v>
       </c>
       <c r="B21" t="s">
         <v>40</v>
       </c>
-      <c r="C21" t="s">
-        <v>8</v>
-      </c>
-      <c r="D21">
+      <c r="C21" s="3" t="str">
+        <f>VLOOKUP(A21&amp;" - "&amp;B21,name6a,2,FALSE)</f>
+        <v>To do</v>
+      </c>
+      <c r="D21" t="s">
+        <v>8</v>
+      </c>
+      <c r="E21">
         <v>2325</v>
       </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>225</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>36</v>
       </c>
       <c r="B22" t="s">
         <v>41</v>
       </c>
-      <c r="C22" t="s">
-        <v>8</v>
-      </c>
-      <c r="D22">
+      <c r="C22" s="3" t="str">
+        <f>VLOOKUP(A22&amp;" - "&amp;B22,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D22" t="s">
+        <v>8</v>
+      </c>
+      <c r="E22">
         <v>2352</v>
       </c>
-      <c r="E22" t="s">
+      <c r="F22" t="s">
         <v>42</v>
       </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>36</v>
       </c>
       <c r="B23" t="s">
         <v>44</v>
       </c>
-      <c r="C23" t="s">
-        <v>8</v>
-      </c>
-      <c r="D23">
+      <c r="C23" s="3" t="str">
+        <f>VLOOKUP(A23&amp;" - "&amp;B23,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D23" t="s">
+        <v>8</v>
+      </c>
+      <c r="E23">
         <v>2343</v>
       </c>
-      <c r="E23" t="s">
+      <c r="F23" t="s">
         <v>45</v>
       </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>47</v>
       </c>
       <c r="B24" t="s">
         <v>48</v>
       </c>
-      <c r="C24" t="s">
-        <v>8</v>
-      </c>
-      <c r="D24">
+      <c r="C24" s="3" t="str">
+        <f>VLOOKUP(A24&amp;" - "&amp;B24,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D24" t="s">
+        <v>8</v>
+      </c>
+      <c r="E24">
         <v>1962</v>
       </c>
-      <c r="E24" t="s">
+      <c r="F24" t="s">
         <v>12</v>
       </c>
-      <c r="F24" t="s">
+      <c r="G24" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>47</v>
       </c>
       <c r="B25" t="s">
         <v>50</v>
       </c>
-      <c r="C25" t="s">
-        <v>8</v>
-      </c>
-      <c r="D25">
+      <c r="C25" s="3" t="str">
+        <f>VLOOKUP(A25&amp;" - "&amp;B25,name6a,2,FALSE)</f>
+        <v>To do</v>
+      </c>
+      <c r="D25" t="s">
+        <v>8</v>
+      </c>
+      <c r="E25">
         <v>1996</v>
       </c>
-      <c r="E25" t="s">
+      <c r="F25" t="s">
         <v>12</v>
       </c>
-      <c r="F25" t="s">
+      <c r="G25" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>51</v>
       </c>
       <c r="B26" t="s">
         <v>51</v>
       </c>
-      <c r="C26" t="s">
-        <v>8</v>
-      </c>
-      <c r="D26">
+      <c r="C26" s="3" t="str">
+        <f>VLOOKUP(A26&amp;" - "&amp;B26,name6a,2,FALSE)</f>
+        <v>tbd</v>
+      </c>
+      <c r="D26" t="s">
+        <v>8</v>
+      </c>
+      <c r="E26">
         <v>2694</v>
       </c>
-      <c r="E26" t="s">
+      <c r="F26" t="s">
         <v>222</v>
       </c>
-      <c r="F26" t="s">
+      <c r="G26" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>51</v>
       </c>
       <c r="B27" t="s">
         <v>52</v>
       </c>
-      <c r="C27" t="s">
-        <v>8</v>
-      </c>
-      <c r="D27">
+      <c r="C27" s="3" t="str">
+        <f>VLOOKUP(A27&amp;" - "&amp;B27,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D27" t="s">
+        <v>8</v>
+      </c>
+      <c r="E27">
         <v>593</v>
       </c>
-      <c r="E27" t="s">
+      <c r="F27" t="s">
         <v>12</v>
       </c>
-      <c r="F27" t="s">
+      <c r="G27" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>54</v>
       </c>
       <c r="B28" t="s">
         <v>55</v>
       </c>
-      <c r="C28" t="s">
-        <v>8</v>
-      </c>
-      <c r="D28">
+      <c r="C28" s="3" t="str">
+        <f>VLOOKUP(A28&amp;" - "&amp;B28,name6a,2,FALSE)</f>
+        <v>To do</v>
+      </c>
+      <c r="D28" t="s">
+        <v>8</v>
+      </c>
+      <c r="E28">
         <v>2802</v>
       </c>
-      <c r="E28" t="s">
+      <c r="F28" t="s">
         <v>81</v>
       </c>
-      <c r="F28" t="s">
+      <c r="G28" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>54</v>
       </c>
       <c r="B29" t="s">
         <v>56</v>
       </c>
-      <c r="C29" t="s">
-        <v>8</v>
-      </c>
-      <c r="D29">
+      <c r="C29" s="3" t="str">
+        <f>VLOOKUP(A29&amp;" - "&amp;B29,name6a,2,FALSE)</f>
+        <v>To do</v>
+      </c>
+      <c r="D29" t="s">
+        <v>8</v>
+      </c>
+      <c r="E29">
         <v>2790</v>
       </c>
-      <c r="E29" t="s">
+      <c r="F29" t="s">
         <v>45</v>
       </c>
-      <c r="F29" t="s">
+      <c r="G29" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>54</v>
       </c>
       <c r="B30" t="s">
         <v>57</v>
       </c>
-      <c r="C30" t="s">
-        <v>8</v>
-      </c>
-      <c r="D30">
+      <c r="C30" s="3" t="str">
+        <f>VLOOKUP(A30&amp;" - "&amp;B30,name6a,2,FALSE)</f>
+        <v>To do</v>
+      </c>
+      <c r="D30" t="s">
+        <v>8</v>
+      </c>
+      <c r="E30">
         <v>2792</v>
       </c>
-      <c r="E30" t="s">
+      <c r="F30" t="s">
         <v>215</v>
       </c>
-      <c r="F30" t="s">
+      <c r="G30" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>54</v>
       </c>
       <c r="B31" t="s">
         <v>58</v>
       </c>
-      <c r="C31" t="s">
-        <v>8</v>
-      </c>
-      <c r="D31">
+      <c r="C31" s="3" t="str">
+        <f>VLOOKUP(A31&amp;" - "&amp;B31,name6a,2,FALSE)</f>
+        <v>To do</v>
+      </c>
+      <c r="D31" t="s">
+        <v>8</v>
+      </c>
+      <c r="E31">
         <v>2791</v>
       </c>
-      <c r="E31" t="s">
+      <c r="F31" t="s">
         <v>215</v>
       </c>
-      <c r="F31" t="s">
+      <c r="G31" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>54</v>
       </c>
       <c r="B32" t="s">
         <v>59</v>
       </c>
-      <c r="C32" t="s">
-        <v>8</v>
-      </c>
-      <c r="D32">
+      <c r="C32" s="3" t="str">
+        <f>VLOOKUP(A32&amp;" - "&amp;B32,name6a,2,FALSE)</f>
+        <v>To do</v>
+      </c>
+      <c r="D32" t="s">
+        <v>8</v>
+      </c>
+      <c r="E32">
         <v>2811</v>
       </c>
-      <c r="E32" t="s">
+      <c r="F32" t="s">
         <v>215</v>
       </c>
-      <c r="F32" t="s">
+      <c r="G32" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>54</v>
       </c>
       <c r="B33" t="s">
         <v>60</v>
       </c>
-      <c r="C33" t="s">
-        <v>8</v>
-      </c>
-      <c r="D33">
+      <c r="C33" s="3" t="str">
+        <f>VLOOKUP(A33&amp;" - "&amp;B33,name6a,2,FALSE)</f>
+        <v>To do</v>
+      </c>
+      <c r="D33" t="s">
+        <v>8</v>
+      </c>
+      <c r="E33">
         <v>2820</v>
       </c>
-      <c r="E33" t="s">
+      <c r="F33" t="s">
         <v>45</v>
       </c>
-      <c r="F33" t="s">
+      <c r="G33" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>54</v>
       </c>
       <c r="B34" t="s">
         <v>61</v>
       </c>
-      <c r="C34" t="s">
-        <v>8</v>
-      </c>
-      <c r="D34">
+      <c r="C34" s="3" t="str">
+        <f>VLOOKUP(A34&amp;" - "&amp;B34,name6a,2,FALSE)</f>
+        <v>To do</v>
+      </c>
+      <c r="D34" t="s">
+        <v>8</v>
+      </c>
+      <c r="E34">
         <v>2819</v>
       </c>
-      <c r="E34" t="s">
+      <c r="F34" t="s">
         <v>215</v>
       </c>
-      <c r="F34" t="s">
+      <c r="G34" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>62</v>
       </c>
       <c r="B35" t="s">
         <v>63</v>
       </c>
-      <c r="C35" t="s">
-        <v>8</v>
-      </c>
-      <c r="D35">
+      <c r="C35" s="3" t="str">
+        <f>VLOOKUP(A35&amp;" - "&amp;B35,name6a,2,FALSE)</f>
+        <v>To do</v>
+      </c>
+      <c r="D35" t="s">
+        <v>8</v>
+      </c>
+      <c r="E35">
         <v>2888</v>
       </c>
-      <c r="E35" t="s">
+      <c r="F35" t="s">
         <v>12</v>
       </c>
-      <c r="F35" t="s">
+      <c r="G35" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>62</v>
       </c>
       <c r="B36" t="s">
         <v>64</v>
       </c>
-      <c r="C36" t="s">
-        <v>8</v>
-      </c>
-      <c r="D36">
+      <c r="C36" s="3" t="str">
+        <f>VLOOKUP(A36&amp;" - "&amp;B36,name6a,2,FALSE)</f>
+        <v>To do</v>
+      </c>
+      <c r="D36" t="s">
+        <v>8</v>
+      </c>
+      <c r="E36">
         <v>2866</v>
       </c>
-      <c r="E36" t="s">
+      <c r="F36" t="s">
         <v>12</v>
       </c>
-      <c r="F36" t="s">
+      <c r="G36" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>62</v>
       </c>
       <c r="B37" t="s">
         <v>65</v>
       </c>
-      <c r="C37" t="s">
-        <v>8</v>
-      </c>
-      <c r="D37">
+      <c r="C37" s="3" t="str">
+        <f>VLOOKUP(A37&amp;" - "&amp;B37,name6a,2,FALSE)</f>
+        <v>To do</v>
+      </c>
+      <c r="D37" t="s">
+        <v>8</v>
+      </c>
+      <c r="E37">
         <v>2866</v>
       </c>
-      <c r="E37" t="s">
+      <c r="F37" t="s">
         <v>12</v>
       </c>
-      <c r="F37" t="s">
+      <c r="G37" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>62</v>
       </c>
       <c r="B38" t="s">
         <v>66</v>
       </c>
-      <c r="C38" t="s">
-        <v>8</v>
-      </c>
-      <c r="D38">
+      <c r="C38" s="3" t="str">
+        <f>VLOOKUP(A38&amp;" - "&amp;B38,name6a,2,FALSE)</f>
+        <v>Mapped</v>
+      </c>
+      <c r="D38" t="s">
+        <v>8</v>
+      </c>
+      <c r="E38">
         <v>2899</v>
       </c>
-      <c r="E38" t="s">
+      <c r="F38" t="s">
         <v>12</v>
       </c>
-      <c r="F38" t="s">
+      <c r="G38" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>67</v>
       </c>
       <c r="B39" t="s">
         <v>67</v>
       </c>
-      <c r="C39" t="s">
-        <v>8</v>
-      </c>
-      <c r="D39">
+      <c r="C39" s="3" t="str">
+        <f>VLOOKUP(A39&amp;" - "&amp;B39,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D39" t="s">
+        <v>8</v>
+      </c>
+      <c r="E39">
         <v>1645</v>
       </c>
-      <c r="E39" t="s">
+      <c r="F39" t="s">
         <v>68</v>
       </c>
-      <c r="F39" t="s">
+      <c r="G39" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>70</v>
       </c>
       <c r="B40" t="s">
         <v>71</v>
       </c>
-      <c r="C40" t="s">
-        <v>8</v>
-      </c>
-      <c r="D40">
+      <c r="C40" s="3" t="str">
+        <f>VLOOKUP(A40&amp;" - "&amp;B40,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D40" t="s">
+        <v>8</v>
+      </c>
+      <c r="E40">
         <v>2061</v>
       </c>
-      <c r="E40" t="s">
+      <c r="F40" t="s">
         <v>72</v>
       </c>
-      <c r="F40" t="s">
+      <c r="G40" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>70</v>
       </c>
       <c r="B41" t="s">
         <v>74</v>
       </c>
-      <c r="C41" t="s">
-        <v>8</v>
-      </c>
-      <c r="D41">
+      <c r="C41" s="3" t="str">
+        <f>VLOOKUP(A41&amp;" - "&amp;B41,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D41" t="s">
+        <v>8</v>
+      </c>
+      <c r="E41">
         <v>2105</v>
       </c>
-      <c r="E41" t="s">
+      <c r="F41" t="s">
         <v>12</v>
       </c>
-      <c r="F41" t="s">
+      <c r="G41" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>70</v>
       </c>
       <c r="B42" t="s">
         <v>76</v>
       </c>
-      <c r="C42" t="s">
-        <v>8</v>
-      </c>
-      <c r="D42">
+      <c r="C42" s="3" t="str">
+        <f>VLOOKUP(A42&amp;" - "&amp;B42,name6a,2,FALSE)</f>
+        <v>Mapped</v>
+      </c>
+      <c r="D42" t="s">
+        <v>8</v>
+      </c>
+      <c r="E42">
         <v>2118</v>
       </c>
-      <c r="E42" t="s">
+      <c r="F42" t="s">
         <v>209</v>
       </c>
-      <c r="F42" t="s">
+      <c r="G42" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>70</v>
       </c>
       <c r="B43" t="s">
         <v>77</v>
       </c>
-      <c r="C43" t="s">
-        <v>8</v>
-      </c>
-      <c r="D43">
+      <c r="C43" s="3" t="str">
+        <f>VLOOKUP(A43&amp;" - "&amp;B43,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D43" t="s">
+        <v>8</v>
+      </c>
+      <c r="E43">
         <v>2126</v>
       </c>
-      <c r="E43" t="s">
+      <c r="F43" t="s">
         <v>78</v>
       </c>
-      <c r="F43" t="s">
+      <c r="G43" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>70</v>
       </c>
       <c r="B44" t="s">
         <v>80</v>
       </c>
-      <c r="C44" t="s">
-        <v>8</v>
-      </c>
-      <c r="D44">
+      <c r="C44" s="3" t="str">
+        <f>VLOOKUP(A44&amp;" - "&amp;B44,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D44" t="s">
+        <v>8</v>
+      </c>
+      <c r="E44">
         <v>2067</v>
       </c>
-      <c r="E44" t="s">
+      <c r="F44" t="s">
         <v>81</v>
       </c>
-      <c r="F44" t="s">
+      <c r="G44" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>70</v>
       </c>
       <c r="B45" t="s">
         <v>83</v>
       </c>
-      <c r="C45" t="s">
-        <v>8</v>
-      </c>
-      <c r="D45">
+      <c r="C45" s="3" t="str">
+        <f>VLOOKUP(A45&amp;" - "&amp;B45,name6a,2,FALSE)</f>
+        <v>Mapped</v>
+      </c>
+      <c r="D45" t="s">
+        <v>8</v>
+      </c>
+      <c r="E45">
         <v>2095</v>
       </c>
-      <c r="E45" t="s">
+      <c r="F45" t="s">
         <v>207</v>
       </c>
-      <c r="F45" t="s">
+      <c r="G45" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>84</v>
       </c>
       <c r="B46" t="s">
         <v>84</v>
       </c>
-      <c r="C46" t="s">
-        <v>8</v>
-      </c>
-      <c r="D46">
+      <c r="C46" s="3" t="str">
+        <f>VLOOKUP(A46&amp;" - "&amp;B46,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D46" t="s">
+        <v>8</v>
+      </c>
+      <c r="E46">
         <v>1042</v>
       </c>
-      <c r="E46" t="s">
+      <c r="F46" t="s">
         <v>68</v>
       </c>
-      <c r="F46" t="s">
+      <c r="G46" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>84</v>
       </c>
       <c r="B47" t="s">
         <v>86</v>
       </c>
-      <c r="C47" t="s">
-        <v>8</v>
-      </c>
-      <c r="D47">
+      <c r="C47" s="3" t="str">
+        <f>VLOOKUP(A47&amp;" - "&amp;B47,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D47" t="s">
+        <v>8</v>
+      </c>
+      <c r="E47">
         <v>1030</v>
       </c>
-      <c r="E47" t="s">
+      <c r="F47" t="s">
         <v>87</v>
       </c>
-      <c r="F47" t="s">
+      <c r="G47" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>84</v>
       </c>
       <c r="B48" t="s">
         <v>89</v>
       </c>
-      <c r="C48" t="s">
-        <v>8</v>
-      </c>
-      <c r="D48">
+      <c r="C48" s="3" t="str">
+        <f>VLOOKUP(A48&amp;" - "&amp;B48,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D48" t="s">
+        <v>8</v>
+      </c>
+      <c r="E48">
         <v>1035</v>
       </c>
-      <c r="E48" t="s">
+      <c r="F48" t="s">
         <v>90</v>
       </c>
-      <c r="F48" t="s">
+      <c r="G48" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>84</v>
       </c>
       <c r="B49" t="s">
         <v>92</v>
       </c>
-      <c r="C49" t="s">
-        <v>8</v>
-      </c>
-      <c r="D49">
+      <c r="C49" s="3" t="str">
+        <f>VLOOKUP(A49&amp;" - "&amp;B49,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D49" t="s">
+        <v>8</v>
+      </c>
+      <c r="E49">
         <v>1116</v>
       </c>
-      <c r="E49" t="s">
+      <c r="F49" t="s">
         <v>12</v>
       </c>
-      <c r="F49" t="s">
+      <c r="G49" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>84</v>
       </c>
       <c r="B50" t="s">
         <v>94</v>
       </c>
-      <c r="C50" t="s">
-        <v>8</v>
-      </c>
-      <c r="D50">
+      <c r="C50" s="3" t="str">
+        <f>VLOOKUP(A50&amp;" - "&amp;B50,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D50" t="s">
+        <v>8</v>
+      </c>
+      <c r="E50">
         <v>1127</v>
       </c>
-      <c r="E50" t="s">
+      <c r="F50" t="s">
         <v>95</v>
       </c>
-      <c r="F50" t="s">
+      <c r="G50" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>96</v>
       </c>
       <c r="B51" t="s">
         <v>97</v>
       </c>
-      <c r="C51" t="s">
-        <v>8</v>
-      </c>
-      <c r="D51">
+      <c r="C51" s="3" t="str">
+        <f>VLOOKUP(A51&amp;" - "&amp;B51,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D51" t="s">
+        <v>8</v>
+      </c>
+      <c r="E51">
         <v>24</v>
       </c>
-      <c r="E51" t="s">
+      <c r="F51" t="s">
         <v>98</v>
       </c>
-      <c r="F51" t="s">
+      <c r="G51" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>96</v>
       </c>
       <c r="B52" t="s">
         <v>100</v>
       </c>
-      <c r="C52" t="s">
-        <v>8</v>
-      </c>
-      <c r="D52">
+      <c r="C52" s="3" t="str">
+        <f>VLOOKUP(A52&amp;" - "&amp;B52,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D52" t="s">
+        <v>8</v>
+      </c>
+      <c r="E52">
         <v>48</v>
       </c>
-      <c r="E52" t="s">
+      <c r="F52" t="s">
         <v>101</v>
       </c>
-      <c r="F52">
+      <c r="G52">
         <v>19470501</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>96</v>
       </c>
       <c r="B53" t="s">
         <v>102</v>
       </c>
-      <c r="C53" t="s">
-        <v>8</v>
-      </c>
-      <c r="D53">
+      <c r="C53" s="3" t="str">
+        <f>VLOOKUP(A53&amp;" - "&amp;B53,name6a,2,FALSE)</f>
+        <v>Mapped</v>
+      </c>
+      <c r="D53" t="s">
+        <v>8</v>
+      </c>
+      <c r="E53">
         <v>30</v>
       </c>
-      <c r="E53" t="s">
+      <c r="F53" t="s">
         <v>114</v>
       </c>
-      <c r="F53" t="s">
+      <c r="G53" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>96</v>
       </c>
       <c r="B54" t="s">
         <v>103</v>
       </c>
-      <c r="C54" t="s">
-        <v>8</v>
-      </c>
-      <c r="D54">
+      <c r="C54" s="3" t="str">
+        <f>VLOOKUP(A54&amp;" - "&amp;B54,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D54" t="s">
+        <v>8</v>
+      </c>
+      <c r="E54">
         <v>53</v>
       </c>
-      <c r="E54" t="s">
+      <c r="F54" t="s">
         <v>104</v>
       </c>
-      <c r="F54" t="s">
+      <c r="G54" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>96</v>
       </c>
       <c r="B55" t="s">
         <v>106</v>
       </c>
-      <c r="C55" t="s">
-        <v>8</v>
-      </c>
-      <c r="D55">
+      <c r="C55" s="3" t="str">
+        <f>VLOOKUP(A55&amp;" - "&amp;B55,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D55" t="s">
+        <v>8</v>
+      </c>
+      <c r="E55">
         <v>39</v>
       </c>
-      <c r="E55" t="s">
+      <c r="F55" t="s">
         <v>107</v>
       </c>
-      <c r="F55" t="s">
+      <c r="G55" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>96</v>
       </c>
       <c r="B56" t="s">
         <v>109</v>
       </c>
-      <c r="C56" t="s">
-        <v>8</v>
-      </c>
-      <c r="D56">
+      <c r="C56" s="3" t="str">
+        <f>VLOOKUP(A56&amp;" - "&amp;B56,name6a,2,FALSE)</f>
+        <v>Omit</v>
+      </c>
+      <c r="D56" t="s">
+        <v>8</v>
+      </c>
+      <c r="E56">
         <v>1886</v>
       </c>
-      <c r="E56" t="s">
+      <c r="F56" t="s">
         <v>12</v>
       </c>
-      <c r="F56" t="s">
+      <c r="G56" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>96</v>
       </c>
       <c r="B57" t="s">
         <v>110</v>
       </c>
-      <c r="C57" t="s">
-        <v>8</v>
-      </c>
-      <c r="D57">
+      <c r="C57" s="3" t="str">
+        <f>VLOOKUP(A57&amp;" - "&amp;B57,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D57" t="s">
+        <v>8</v>
+      </c>
+      <c r="E57">
         <v>40</v>
       </c>
-      <c r="E57" t="s">
+      <c r="F57" t="s">
         <v>111</v>
       </c>
-      <c r="F57" t="s">
+      <c r="G57" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>96</v>
       </c>
       <c r="B58" t="s">
         <v>113</v>
       </c>
-      <c r="C58" t="s">
-        <v>8</v>
-      </c>
-      <c r="D58">
+      <c r="C58" s="3" t="str">
+        <f>VLOOKUP(A58&amp;" - "&amp;B58,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D58" t="s">
+        <v>8</v>
+      </c>
+      <c r="E58">
         <v>29</v>
       </c>
-      <c r="E58" t="s">
+      <c r="F58" t="s">
         <v>114</v>
       </c>
-      <c r="F58" t="s">
+      <c r="G58" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>96</v>
       </c>
       <c r="B59" t="s">
         <v>116</v>
       </c>
-      <c r="C59" t="s">
-        <v>8</v>
-      </c>
-      <c r="D59">
+      <c r="C59" s="3" t="str">
+        <f>VLOOKUP(A59&amp;" - "&amp;B59,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D59" t="s">
+        <v>8</v>
+      </c>
+      <c r="E59">
         <v>29</v>
       </c>
-      <c r="E59" t="s">
+      <c r="F59" t="s">
         <v>117</v>
       </c>
-      <c r="F59" t="s">
+      <c r="G59" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>96</v>
       </c>
       <c r="B60" t="s">
         <v>119</v>
       </c>
-      <c r="C60" t="s">
-        <v>8</v>
-      </c>
-      <c r="D60">
+      <c r="C60" s="3" t="str">
+        <f>VLOOKUP(A60&amp;" - "&amp;B60,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D60" t="s">
+        <v>8</v>
+      </c>
+      <c r="E60">
         <v>86</v>
       </c>
-      <c r="E60" t="s">
+      <c r="F60" t="s">
         <v>120</v>
       </c>
-      <c r="F60" t="s">
+      <c r="G60" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>96</v>
       </c>
       <c r="B61" t="s">
         <v>122</v>
       </c>
-      <c r="C61" t="s">
-        <v>8</v>
-      </c>
-      <c r="D61">
+      <c r="C61" s="3" t="str">
+        <f>VLOOKUP(A61&amp;" - "&amp;B61,name6a,2,FALSE)</f>
+        <v>To do</v>
+      </c>
+      <c r="D61" t="s">
+        <v>8</v>
+      </c>
+      <c r="E61">
         <v>32</v>
       </c>
-      <c r="E61" t="s">
+      <c r="F61" t="s">
         <v>203</v>
       </c>
-      <c r="F61" t="s">
+      <c r="G61" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>96</v>
       </c>
       <c r="B62" t="s">
         <v>123</v>
       </c>
-      <c r="C62" t="s">
-        <v>8</v>
-      </c>
-      <c r="D62">
+      <c r="C62" s="3" t="str">
+        <f>VLOOKUP(A62&amp;" - "&amp;B62,name6a,2,FALSE)</f>
+        <v>To do</v>
+      </c>
+      <c r="D62" t="s">
+        <v>8</v>
+      </c>
+      <c r="E62">
         <v>44</v>
       </c>
-      <c r="E62" t="s">
+      <c r="F62" t="s">
         <v>201</v>
       </c>
-      <c r="F62" t="s">
+      <c r="G62" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>96</v>
       </c>
       <c r="B63" t="s">
         <v>124</v>
       </c>
-      <c r="C63" t="s">
-        <v>8</v>
-      </c>
-      <c r="D63">
+      <c r="C63" s="3" t="str">
+        <f>VLOOKUP(A63&amp;" - "&amp;B63,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D63" t="s">
+        <v>8</v>
+      </c>
+      <c r="E63">
         <v>51</v>
       </c>
-      <c r="E63" t="s">
+      <c r="F63" t="s">
         <v>125</v>
       </c>
-      <c r="F63" t="s">
+      <c r="G63" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>96</v>
       </c>
       <c r="B64" t="s">
         <v>127</v>
       </c>
-      <c r="C64" t="s">
-        <v>8</v>
-      </c>
-      <c r="D64">
+      <c r="C64" s="3" t="str">
+        <f>VLOOKUP(A64&amp;" - "&amp;B64,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D64" t="s">
+        <v>8</v>
+      </c>
+      <c r="E64">
         <v>68</v>
       </c>
-      <c r="E64" t="s">
+      <c r="F64" t="s">
         <v>128</v>
       </c>
-      <c r="F64" t="s">
+      <c r="G64" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>96</v>
       </c>
       <c r="B65" t="s">
         <v>130</v>
       </c>
-      <c r="C65" t="s">
-        <v>8</v>
-      </c>
-      <c r="D65">
+      <c r="C65" s="3" t="str">
+        <f>VLOOKUP(A65&amp;" - "&amp;B65,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D65" t="s">
+        <v>8</v>
+      </c>
+      <c r="E65">
         <v>57</v>
       </c>
-      <c r="E65" t="s">
+      <c r="F65" t="s">
         <v>45</v>
       </c>
-      <c r="F65" t="s">
+      <c r="G65" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>96</v>
       </c>
       <c r="B66" t="s">
         <v>132</v>
       </c>
-      <c r="C66" t="s">
-        <v>8</v>
-      </c>
-      <c r="D66">
+      <c r="C66" s="3" t="str">
+        <f>VLOOKUP(A66&amp;" - "&amp;B66,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D66" t="s">
+        <v>8</v>
+      </c>
+      <c r="E66">
         <v>47</v>
       </c>
-      <c r="E66" t="s">
+      <c r="F66" t="s">
         <v>133</v>
       </c>
-      <c r="F66" t="s">
+      <c r="G66" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>96</v>
       </c>
       <c r="B67" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="C67" s="3" t="str">
+        <f>VLOOKUP(A67&amp;" - "&amp;B67,name6a,2,FALSE)</f>
+        <v>Omit</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>96</v>
       </c>
       <c r="B68" t="s">
         <v>136</v>
       </c>
-      <c r="C68" t="s">
-        <v>8</v>
-      </c>
-      <c r="D68">
+      <c r="C68" s="3" t="str">
+        <f>VLOOKUP(A68&amp;" - "&amp;B68,name6a,2,FALSE)</f>
+        <v>Omit</v>
+      </c>
+      <c r="D68" t="s">
+        <v>8</v>
+      </c>
+      <c r="E68">
         <v>1897</v>
       </c>
-      <c r="E68" t="s">
+      <c r="F68" t="s">
         <v>12</v>
       </c>
-      <c r="F68" t="s">
+      <c r="G68" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>96</v>
       </c>
       <c r="B69" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="C69" s="3" t="str">
+        <f>VLOOKUP(A69&amp;" - "&amp;B69,name6a,2,FALSE)</f>
+        <v>Mapped</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>96</v>
       </c>
       <c r="B70" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="C70" s="3" t="str">
+        <f>VLOOKUP(A70&amp;" - "&amp;B70,name6a,2,FALSE)</f>
+        <v>To do</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>139</v>
       </c>
       <c r="B71" t="s">
         <v>139</v>
       </c>
-      <c r="C71" t="s">
-        <v>8</v>
-      </c>
-      <c r="D71">
+      <c r="C71" s="3" t="str">
+        <f>VLOOKUP(A71&amp;" - "&amp;B71,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D71" t="s">
+        <v>8</v>
+      </c>
+      <c r="E71">
         <v>336</v>
       </c>
-      <c r="E71" t="s">
+      <c r="F71" t="s">
         <v>12</v>
       </c>
-      <c r="F71" t="s">
+      <c r="G71" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>139</v>
       </c>
       <c r="B72" t="s">
         <v>141</v>
       </c>
-      <c r="C72" t="s">
-        <v>8</v>
-      </c>
-      <c r="D72">
+      <c r="C72" s="3" t="str">
+        <f>VLOOKUP(A72&amp;" - "&amp;B72,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D72" t="s">
+        <v>8</v>
+      </c>
+      <c r="E72">
         <v>636</v>
       </c>
-      <c r="E72" t="s">
+      <c r="F72" t="s">
         <v>27</v>
       </c>
-      <c r="F72" t="s">
+      <c r="G72" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>139</v>
       </c>
       <c r="B73" t="s">
         <v>143</v>
       </c>
-      <c r="C73" t="s">
-        <v>8</v>
-      </c>
-      <c r="D73">
+      <c r="C73" s="3" t="str">
+        <f>VLOOKUP(A73&amp;" - "&amp;B73,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D73" t="s">
+        <v>8</v>
+      </c>
+      <c r="E73">
         <v>527</v>
       </c>
-      <c r="E73" t="s">
+      <c r="F73" t="s">
         <v>144</v>
       </c>
-      <c r="F73" t="s">
+      <c r="G73" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>146</v>
       </c>
       <c r="B74" t="s">
         <v>146</v>
       </c>
-      <c r="C74" t="s">
-        <v>8</v>
-      </c>
-      <c r="D74">
+      <c r="C74" s="3" t="str">
+        <f>VLOOKUP(A74&amp;" - "&amp;B74,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D74" t="s">
+        <v>8</v>
+      </c>
+      <c r="E74">
         <v>1335</v>
       </c>
-      <c r="E74" t="s">
+      <c r="F74" t="s">
         <v>147</v>
       </c>
-      <c r="F74" t="s">
+      <c r="G74" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>146</v>
       </c>
       <c r="B75" t="s">
         <v>149</v>
       </c>
-      <c r="C75" t="s">
-        <v>8</v>
-      </c>
-      <c r="D75">
+      <c r="C75" s="3" t="str">
+        <f>VLOOKUP(A75&amp;" - "&amp;B75,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D75" t="s">
+        <v>8</v>
+      </c>
+      <c r="E75">
         <v>1538</v>
       </c>
-      <c r="E75" t="s">
+      <c r="F75" t="s">
         <v>147</v>
       </c>
-      <c r="F75" t="s">
+      <c r="G75" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>146</v>
       </c>
       <c r="B76" t="s">
         <v>151</v>
       </c>
-      <c r="C76" t="s">
-        <v>8</v>
-      </c>
-      <c r="D76">
+      <c r="C76" s="3" t="str">
+        <f>VLOOKUP(A76&amp;" - "&amp;B76,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D76" t="s">
+        <v>8</v>
+      </c>
+      <c r="E76">
         <v>1344</v>
       </c>
-      <c r="E76" t="s">
+      <c r="F76" t="s">
         <v>42</v>
       </c>
-      <c r="F76" t="s">
+      <c r="G76" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>146</v>
       </c>
       <c r="B77" t="s">
         <v>153</v>
       </c>
-      <c r="C77" t="s">
-        <v>8</v>
-      </c>
-      <c r="D77">
+      <c r="C77" s="3" t="str">
+        <f>VLOOKUP(A77&amp;" - "&amp;B77,name6a,2,FALSE)</f>
+        <v>To do</v>
+      </c>
+      <c r="D77" t="s">
+        <v>8</v>
+      </c>
+      <c r="E77">
         <v>2911</v>
       </c>
-      <c r="E77" t="s">
+      <c r="F77" t="s">
         <v>27</v>
       </c>
-      <c r="F77" t="s">
+      <c r="G77" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>154</v>
       </c>
       <c r="B78" t="s">
         <v>155</v>
       </c>
-      <c r="C78" t="s">
-        <v>8</v>
-      </c>
-      <c r="D78">
+      <c r="C78" s="3" t="str">
+        <f>VLOOKUP(A78&amp;" - "&amp;B78,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D78" t="s">
+        <v>8</v>
+      </c>
+      <c r="E78">
         <v>120</v>
       </c>
-      <c r="E78" t="s">
+      <c r="F78" t="s">
         <v>156</v>
       </c>
-      <c r="F78" t="s">
+      <c r="G78" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>154</v>
       </c>
       <c r="B79" t="s">
         <v>158</v>
       </c>
-      <c r="C79" t="s">
-        <v>8</v>
-      </c>
-      <c r="D79">
+      <c r="C79" s="3" t="str">
+        <f>VLOOKUP(A79&amp;" - "&amp;B79,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D79" t="s">
+        <v>8</v>
+      </c>
+      <c r="E79">
         <v>94</v>
       </c>
-      <c r="E79" t="s">
+      <c r="F79" t="s">
         <v>159</v>
       </c>
-      <c r="F79" t="s">
+      <c r="G79" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>154</v>
       </c>
       <c r="B80" t="s">
         <v>161</v>
       </c>
-      <c r="C80" t="s">
-        <v>8</v>
-      </c>
-      <c r="D80">
+      <c r="C80" s="3" t="str">
+        <f>VLOOKUP(A80&amp;" - "&amp;B80,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D80" t="s">
+        <v>8</v>
+      </c>
+      <c r="E80">
         <v>110</v>
       </c>
-      <c r="E80" t="s">
+      <c r="F80" t="s">
         <v>45</v>
       </c>
-      <c r="F80" t="s">
+      <c r="G80" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>154</v>
       </c>
       <c r="B81" t="s">
         <v>163</v>
       </c>
-      <c r="C81" t="s">
-        <v>8</v>
-      </c>
-      <c r="D81">
+      <c r="C81" s="3" t="str">
+        <f>VLOOKUP(A81&amp;" - "&amp;B81,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D81" t="s">
+        <v>8</v>
+      </c>
+      <c r="E81">
         <v>106</v>
       </c>
-      <c r="E81" t="s">
+      <c r="F81" t="s">
         <v>164</v>
       </c>
-      <c r="F81" t="s">
+      <c r="G81" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>166</v>
       </c>
       <c r="B82" t="s">
         <v>166</v>
       </c>
-      <c r="C82" t="s">
-        <v>8</v>
-      </c>
-      <c r="D82">
+      <c r="C82" s="3" t="str">
+        <f>VLOOKUP(A82&amp;" - "&amp;B82,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D82" t="s">
+        <v>8</v>
+      </c>
+      <c r="E82">
         <v>1862</v>
       </c>
-      <c r="E82" t="s">
+      <c r="F82" t="s">
         <v>12</v>
       </c>
-      <c r="F82" t="s">
+      <c r="G82" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>166</v>
       </c>
       <c r="B83" t="s">
         <v>168</v>
       </c>
-      <c r="C83" t="s">
-        <v>8</v>
-      </c>
-      <c r="D83">
+      <c r="C83" s="3" t="str">
+        <f>VLOOKUP(A83&amp;" - "&amp;B83,name6a,2,FALSE)</f>
+        <v>Later</v>
+      </c>
+      <c r="D83" t="s">
+        <v>8</v>
+      </c>
+      <c r="E83">
         <v>1908</v>
       </c>
-      <c r="E83" t="s">
+      <c r="F83" t="s">
         <v>12</v>
       </c>
-      <c r="F83" t="s">
+      <c r="G83" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>169</v>
       </c>
       <c r="B84" t="s">
         <v>170</v>
       </c>
-      <c r="C84" t="s">
-        <v>8</v>
-      </c>
-      <c r="D84">
+      <c r="C84" s="3" t="str">
+        <f>VLOOKUP(A84&amp;" - "&amp;B84,name6a,2,FALSE)</f>
+        <v>Yes</v>
+      </c>
+      <c r="D84" t="s">
+        <v>8</v>
+      </c>
+      <c r="E84">
         <v>1456</v>
       </c>
-      <c r="E84" t="s">
+      <c r="F84" t="s">
         <v>9</v>
       </c>
-      <c r="F84" t="s">
+      <c r="G84" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>172</v>
       </c>
       <c r="B85" t="s">
         <v>173</v>
       </c>
-      <c r="C85" t="s">
-        <v>8</v>
-      </c>
-      <c r="D85">
+      <c r="C85" s="3" t="str">
+        <f>VLOOKUP(A85&amp;" - "&amp;B85,name6a,2,FALSE)</f>
+        <v>Mapped</v>
+      </c>
+      <c r="D85" t="s">
+        <v>8</v>
+      </c>
+      <c r="E85">
         <v>2241</v>
       </c>
-      <c r="E85" t="s">
+      <c r="F85" t="s">
         <v>12</v>
       </c>
-      <c r="F85" t="s">
+      <c r="G85" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>172</v>
       </c>
       <c r="B86" t="s">
         <v>174</v>
       </c>
-      <c r="C86" t="s">
-        <v>8</v>
-      </c>
-      <c r="D86">
+      <c r="C86" s="3" t="str">
+        <f>VLOOKUP(A86&amp;" - "&amp;B86,name6a,2,FALSE)</f>
+        <v>Mapped</v>
+      </c>
+      <c r="D86" t="s">
+        <v>8</v>
+      </c>
+      <c r="E86">
         <v>2205</v>
       </c>
-      <c r="E86" t="s">
+      <c r="F86" t="s">
         <v>12</v>
       </c>
-      <c r="F86" t="s">
+      <c r="G86" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>172</v>
       </c>
       <c r="B87" t="s">
         <v>175</v>
       </c>
-      <c r="C87" t="s">
-        <v>8</v>
-      </c>
-      <c r="D87">
+      <c r="C87" s="3" t="str">
+        <f>VLOOKUP(A87&amp;" - "&amp;B87,name6a,2,FALSE)</f>
+        <v>Mapped</v>
+      </c>
+      <c r="D87" t="s">
+        <v>8</v>
+      </c>
+      <c r="E87">
         <v>2193</v>
       </c>
-      <c r="E87" t="s">
+      <c r="F87" t="s">
         <v>12</v>
       </c>
-      <c r="F87" t="s">
+      <c r="G87" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>172</v>
       </c>
       <c r="B88" t="s">
         <v>176</v>
       </c>
-      <c r="C88" t="s">
-        <v>8</v>
-      </c>
-      <c r="D88">
+      <c r="C88" s="3" t="str">
+        <f>VLOOKUP(A88&amp;" - "&amp;B88,name6a,2,FALSE)</f>
+        <v>Mapped</v>
+      </c>
+      <c r="D88" t="s">
+        <v>8</v>
+      </c>
+      <c r="E88">
         <v>2217</v>
       </c>
-      <c r="E88" t="s">
+      <c r="F88" t="s">
         <v>12</v>
       </c>
-      <c r="F88" t="s">
+      <c r="G88" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>172</v>
       </c>
       <c r="B89" t="s">
         <v>177</v>
       </c>
-      <c r="C89" t="s">
-        <v>8</v>
-      </c>
-      <c r="D89">
+      <c r="C89" s="3" t="str">
+        <f>VLOOKUP(A89&amp;" - "&amp;B89,name6a,2,FALSE)</f>
+        <v>Mapped</v>
+      </c>
+      <c r="D89" t="s">
+        <v>8</v>
+      </c>
+      <c r="E89">
         <v>2253</v>
       </c>
-      <c r="E89" t="s">
+      <c r="F89" t="s">
         <v>12</v>
       </c>
-      <c r="F89" t="s">
+      <c r="G89" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>172</v>
       </c>
       <c r="B90" t="s">
         <v>178</v>
       </c>
-      <c r="C90" t="s">
-        <v>8</v>
-      </c>
-      <c r="D90">
+      <c r="C90" s="3" t="str">
+        <f>VLOOKUP(A90&amp;" - "&amp;B90,name6a,2,FALSE)</f>
+        <v>Mapped</v>
+      </c>
+      <c r="D90" t="s">
+        <v>8</v>
+      </c>
+      <c r="E90">
         <v>2229</v>
       </c>
-      <c r="E90" t="s">
+      <c r="F90" t="s">
         <v>12</v>
       </c>
-      <c r="F90" t="s">
+      <c r="G90" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>172</v>
       </c>
       <c r="B91" t="s">
         <v>179</v>
       </c>
-      <c r="C91" t="s">
-        <v>8</v>
-      </c>
-      <c r="D91">
+      <c r="C91" s="3" t="str">
+        <f>VLOOKUP(A91&amp;" - "&amp;B91,name6a,2,FALSE)</f>
+        <v>Mapped</v>
+      </c>
+      <c r="D91" t="s">
+        <v>8</v>
+      </c>
+      <c r="E91">
         <v>2178</v>
       </c>
-      <c r="E91" t="s">
+      <c r="F91" t="s">
         <v>12</v>
       </c>
-      <c r="F91" t="s">
+      <c r="G91" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>172</v>
       </c>
       <c r="B92" t="s">
         <v>181</v>
       </c>
-      <c r="C92" t="s">
-        <v>8</v>
-      </c>
-      <c r="D92">
+      <c r="C92" s="3" t="str">
+        <f>VLOOKUP(A92&amp;" - "&amp;B92,name6a,2,FALSE)</f>
+        <v>Mapped</v>
+      </c>
+      <c r="D92" t="s">
+        <v>8</v>
+      </c>
+      <c r="E92">
         <v>2289</v>
       </c>
-      <c r="E92" t="s">
+      <c r="F92" t="s">
         <v>12</v>
       </c>
-      <c r="F92" t="s">
+      <c r="G92" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>172</v>
       </c>
       <c r="B93" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="C93" s="3" t="str">
+        <f>VLOOKUP(A93&amp;" - "&amp;B93,name6a,2,FALSE)</f>
+        <v>Mapped</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>172</v>
       </c>
       <c r="B94" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="C94" s="3" t="str">
+        <f>VLOOKUP(A94&amp;" - "&amp;B94,name6a,2,FALSE)</f>
+        <v>Mapped</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>172</v>
       </c>
       <c r="B95" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="C95" s="3" t="str">
+        <f>VLOOKUP(A95&amp;" - "&amp;B95,name6a,2,FALSE)</f>
+        <v>Mapped</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>172</v>
       </c>
       <c r="B96" t="s">
         <v>185</v>
       </c>
-      <c r="C96" t="s">
-        <v>8</v>
-      </c>
-      <c r="D96">
+      <c r="C96" s="3" t="str">
+        <f>VLOOKUP(A96&amp;" - "&amp;B96,name6a,2,FALSE)</f>
+        <v>Mapped</v>
+      </c>
+      <c r="D96" t="s">
+        <v>8</v>
+      </c>
+      <c r="E96">
         <v>2277</v>
       </c>
-      <c r="E96" t="s">
+      <c r="F96" t="s">
         <v>12</v>
       </c>
-      <c r="F96" t="s">
+      <c r="G96" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>172</v>
       </c>
       <c r="B97" t="s">
         <v>186</v>
       </c>
-      <c r="C97" t="s">
-        <v>8</v>
-      </c>
-      <c r="D97">
+      <c r="C97" s="3" t="str">
+        <f>VLOOKUP(A97&amp;" - "&amp;B97,name6a,2,FALSE)</f>
+        <v>Mapped</v>
+      </c>
+      <c r="D97" t="s">
+        <v>8</v>
+      </c>
+      <c r="E97">
         <v>2265</v>
       </c>
-      <c r="E97" t="s">
+      <c r="F97" t="s">
         <v>12</v>
       </c>
-      <c r="F97" t="s">
+      <c r="G97" t="s">
         <v>187</v>
       </c>
     </row>

</xml_diff>

<commit_message>
correct line numbers in audit file
</commit_message>
<xml_diff>
--- a/CDAtoFHIRExamples/Input/USCDI_v3_Myra_compare.xlsx
+++ b/CDAtoFHIRExamples/Input/USCDI_v3_Myra_compare.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repos\CCDAtoFHIRSamples\CDAtoFHIRExamples\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6552BFC3-6157-4B2D-8C5D-EF0B87D11EAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE42287E-B6C6-4AF6-86A7-EEA5AE39EA4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{AD9AA5AD-85CE-4E99-8021-1D0325A3266B}"/>
   </bookViews>
   <sheets>
     <sheet name="USCDI_v3_Myra_v6" sheetId="1" r:id="rId1"/>
-    <sheet name="USCDI_v3_Myra_v7" sheetId="2" r:id="rId2"/>
+    <sheet name="USCDI_v3_Myra_v7" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="name6">USCDI_v3_Myra_v6!$C:$C</definedName>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="855" uniqueCount="260">
   <si>
     <t>USCDI Data Class</t>
   </si>
@@ -649,9 +649,6 @@
     <t>742 Evergreen Terrace, Portland, OR 97201</t>
   </si>
   <si>
-    <t>addr use=OLD</t>
-  </si>
-  <si>
     <t>446141000124107 Identifies as female gender</t>
   </si>
   <si>
@@ -670,18 +667,6 @@
     <t>interpretationCode</t>
   </si>
   <si>
-    <t>82810-3 Not pregnant</t>
-  </si>
-  <si>
-    <t>Cognitive function - Alert and oriented x3</t>
-  </si>
-  <si>
-    <t>54522-8 Functional status - Independent</t>
-  </si>
-  <si>
-    <t>96867-5 Disability status - No</t>
-  </si>
-  <si>
     <t>1EG4-TE5-MK72</t>
   </si>
   <si>
@@ -697,24 +682,12 @@
     <t>GRP-98765</t>
   </si>
   <si>
-    <t>MA Medicare Part A</t>
-  </si>
-  <si>
-    <t>active</t>
-  </si>
-  <si>
     <t>75310-3 Health Concern Act</t>
   </si>
   <si>
     <t>section/act</t>
   </si>
   <si>
-    <t>410518001 Adequate food supply</t>
-  </si>
-  <si>
-    <t>Urgent Care Center, Portland, OR</t>
-  </si>
-  <si>
     <t>participant LOC</t>
   </si>
   <si>
@@ -781,10 +754,70 @@
     <t>tbd</t>
   </si>
   <si>
-    <t>Omit</t>
-  </si>
-  <si>
     <t>Found in Myra6</t>
+  </si>
+  <si>
+    <t>1191 Aspirin; 762952008 Peanut (line 925)</t>
+  </si>
+  <si>
+    <t>Community Urgent Care, 1004 Healthcare Dr., Portland, OR</t>
+  </si>
+  <si>
+    <t>99213 Office/outpatient established low MDM 20-29 min</t>
+  </si>
+  <si>
+    <t>observation moodCode=GOL</t>
+  </si>
+  <si>
+    <t>262285001 Weight decreased (finding)</t>
+  </si>
+  <si>
+    <t>1078229009 Food security</t>
+  </si>
+  <si>
+    <t>completed (Coverage Activity)</t>
+  </si>
+  <si>
+    <t>1 Medicare (Source of Payment Typology); narrative: Medicare Part A</t>
+  </si>
+  <si>
+    <t>89571-4 Disability status (LA29240-1 No identified disability)</t>
+  </si>
+  <si>
+    <t>54522-8 Functional status (371153006 Independent)</t>
+  </si>
+  <si>
+    <t>373930000 Cognitive function finding (66557003 No impairment)</t>
+  </si>
+  <si>
+    <t>82810-3 Pregnancy status (60001007 Not pregnant)</t>
+  </si>
+  <si>
+    <t>CVX 88 Influenza; CVX 43 Hepatitis B (line 1779)</t>
+  </si>
+  <si>
+    <t>1190220 Albuterol/ipratropium; 1657066 Bevacizumab (line 1237)</t>
+  </si>
+  <si>
+    <t>56018004 Wheezing; 363406005 Malignant neoplasm of colon (line 1264)</t>
+  </si>
+  <si>
+    <t>addr use=BAD</t>
+  </si>
+  <si>
+    <t>99501-9 Female-typical parameter (LA32969-2)</t>
+  </si>
+  <si>
+    <t>233604007 Pneumonia; 195967001 Asthma (line 456); 414916001 Obesity (line 668); etc.</t>
+  </si>
+  <si>
+    <t>20140405235959 Acute pharyngitis resolution</t>
+  </si>
+  <si>
+    <t>416940007 Chest x-ray; 73761001 Colonoscopy (line 1440); 33206 Pacemaker (line 1563); etc.</t>
+  </si>
+  <si>
+    <t>Colonoscope UDI (line 1454); Pacemaker UDI (line 1568)</t>
   </si>
 </sst>
 </file>
@@ -1674,7 +1707,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>244</v>
+        <v>235</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -1797,7 +1830,7 @@
         <v>Care Team Member(s) - Care Team Member Name</v>
       </c>
       <c r="D6" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
@@ -1812,7 +1845,7 @@
         <v>Care Team Member(s) - Care Team Member Identifier</v>
       </c>
       <c r="D7" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
@@ -1827,7 +1860,7 @@
         <v>Care Team Member(s) - Care Team Member Location</v>
       </c>
       <c r="D8" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
@@ -1842,7 +1875,7 @@
         <v>Care Team Member(s) - Care Team Member Telecom</v>
       </c>
       <c r="D9" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
@@ -1857,7 +1890,7 @@
         <v>Care Team Member(s) - Care Team Member Role</v>
       </c>
       <c r="D10" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
@@ -1896,7 +1929,7 @@
         <v>Clinical Notes - Discharge Summary Note</v>
       </c>
       <c r="D12" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
@@ -1911,7 +1944,7 @@
         <v>Clinical Notes - History &amp; Physical</v>
       </c>
       <c r="D13" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
@@ -1926,7 +1959,7 @@
         <v>Clinical Notes - Imaging Narrative</v>
       </c>
       <c r="D14" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
@@ -1941,7 +1974,7 @@
         <v>Clinical Notes - Laboratory Report Narrative</v>
       </c>
       <c r="D15" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
@@ -1956,7 +1989,7 @@
         <v>Clinical Notes - Pathology Report Narrative</v>
       </c>
       <c r="D16" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
@@ -1971,7 +2004,7 @@
         <v>Clinical Notes - Procedure Note</v>
       </c>
       <c r="D17" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
@@ -1986,7 +2019,7 @@
         <v>Clinical Notes - Progress Note</v>
       </c>
       <c r="D18" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
@@ -2025,7 +2058,7 @@
         <v>Encounter Information - Encounter Disposition</v>
       </c>
       <c r="D20" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
@@ -2040,7 +2073,7 @@
         <v>Encounter Information - Encounter Location</v>
       </c>
       <c r="D21" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
@@ -2127,7 +2160,7 @@
         <v>Goals - SDOH Goals</v>
       </c>
       <c r="D25" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
@@ -2142,7 +2175,7 @@
         <v>Health Concerns - Health Concerns</v>
       </c>
       <c r="D26" t="s">
-        <v>246</v>
+        <v>237</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
@@ -2181,7 +2214,7 @@
         <v>Health Insurance Information - Coverage Status</v>
       </c>
       <c r="D28" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
@@ -2196,7 +2229,7 @@
         <v>Health Insurance Information - Coverage Type</v>
       </c>
       <c r="D29" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.35">
@@ -2211,7 +2244,7 @@
         <v>Health Insurance Information - Group Identifier</v>
       </c>
       <c r="D30" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
@@ -2226,7 +2259,7 @@
         <v>Health Insurance Information - Member Identifier</v>
       </c>
       <c r="D31" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
@@ -2241,7 +2274,7 @@
         <v>Health Insurance Information - Payer Identifier</v>
       </c>
       <c r="D32" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
@@ -2256,7 +2289,7 @@
         <v>Health Insurance Information - Relationship to Subscriber</v>
       </c>
       <c r="D33" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
@@ -2271,7 +2304,7 @@
         <v>Health Insurance Information - Subscriber Identifier</v>
       </c>
       <c r="D34" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
@@ -2286,7 +2319,7 @@
         <v>Health Status/Assessments - Disability Status</v>
       </c>
       <c r="D35" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
@@ -2301,7 +2334,7 @@
         <v>Health Status/Assessments - Functional Status</v>
       </c>
       <c r="D36" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
@@ -2316,7 +2349,7 @@
         <v>Health Status/Assessments - Mental/Cognitive Status</v>
       </c>
       <c r="D37" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
@@ -2331,7 +2364,7 @@
         <v>Health Status/Assessments - Pregnancy Status</v>
       </c>
       <c r="D38" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.35">
@@ -2418,7 +2451,7 @@
         <v>Laboratory - Result Interpretation</v>
       </c>
       <c r="D42" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
@@ -2481,7 +2514,7 @@
         <v>Laboratory - Specimen Type</v>
       </c>
       <c r="D45" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.35">
@@ -2664,7 +2697,7 @@
         <v>Patient Demographics/Information - Email Address</v>
       </c>
       <c r="D53" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.35">
@@ -2727,7 +2760,7 @@
         <v>Patient Demographics/Information - Gender Identity</v>
       </c>
       <c r="D56" t="s">
-        <v>247</v>
+        <v>234</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.35">
@@ -2838,7 +2871,7 @@
         <v>Patient Demographics/Information - Previous Address</v>
       </c>
       <c r="D61" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.35">
@@ -2853,7 +2886,7 @@
         <v>Patient Demographics/Information - Previous Name</v>
       </c>
       <c r="D62" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.35">
@@ -2964,7 +2997,7 @@
         <v>Patient Demographics/Information - Sex Parameter for Clinical Use</v>
       </c>
       <c r="D67" t="s">
-        <v>247</v>
+        <v>234</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.35">
@@ -2979,7 +3012,7 @@
         <v>Patient Demographics/Information - Sexual Orientation</v>
       </c>
       <c r="D68" t="s">
-        <v>247</v>
+        <v>234</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.35">
@@ -2994,7 +3027,7 @@
         <v>Patient Demographics/Information - Suffix</v>
       </c>
       <c r="D69" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.35">
@@ -3009,7 +3042,7 @@
         <v>Patient Demographics/Information - Tribal Affiliation</v>
       </c>
       <c r="D70" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.35">
@@ -3168,7 +3201,7 @@
         <v>Procedures - Reason for Referral</v>
       </c>
       <c r="D77" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.35">
@@ -3303,7 +3336,7 @@
         <v>Smoking Status - Substance Use</v>
       </c>
       <c r="D83" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.35">
@@ -3342,7 +3375,7 @@
         <v>Vital Signs - BMI</v>
       </c>
       <c r="D85" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.35">
@@ -3357,7 +3390,7 @@
         <v>Vital Signs - Blood Pressure (Diastolic)</v>
       </c>
       <c r="D86" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.35">
@@ -3372,7 +3405,7 @@
         <v>Vital Signs - Blood Pressure (Systolic)</v>
       </c>
       <c r="D87" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.35">
@@ -3387,7 +3420,7 @@
         <v>Vital Signs - Body Height</v>
       </c>
       <c r="D88" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.35">
@@ -3402,7 +3435,7 @@
         <v>Vital Signs - Body Temperature</v>
       </c>
       <c r="D89" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.35">
@@ -3417,7 +3450,7 @@
         <v>Vital Signs - Body Weight</v>
       </c>
       <c r="D90" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.35">
@@ -3432,7 +3465,7 @@
         <v>Vital Signs - Heart Rate</v>
       </c>
       <c r="D91" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
       <c r="E91">
         <v>2114</v>
@@ -3456,7 +3489,7 @@
         <v>Vital Signs - Inhaled Oxygen Concentration</v>
       </c>
       <c r="D92" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.35">
@@ -3471,7 +3504,7 @@
         <v>Vital Signs - Pediatric BMI for Age</v>
       </c>
       <c r="D93" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.35">
@@ -3486,7 +3519,7 @@
         <v>Vital Signs - Pediatric Head Circumference</v>
       </c>
       <c r="D94" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.35">
@@ -3501,7 +3534,7 @@
         <v>Vital Signs - Pediatric Weight for Height</v>
       </c>
       <c r="D95" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.35">
@@ -3516,7 +3549,7 @@
         <v>Vital Signs - Pulse Oximetry</v>
       </c>
       <c r="D96" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.35">
@@ -3531,7 +3564,7 @@
         <v>Vital Signs - Respiratory Rate</v>
       </c>
       <c r="D97" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
     </row>
   </sheetData>
@@ -3540,16 +3573,12 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4C70803-C6D0-4941-8F3C-8CF7B7FD09A5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AAE02FC-7CCE-48B3-ADBC-27BF65697042}">
   <dimension ref="A1:G97"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29" style="3" customWidth="1"/>
-    <col min="4" max="4" width="10.90625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="26.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="59.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
@@ -3560,7 +3589,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -3583,7 +3612,7 @@
         <v>7</v>
       </c>
       <c r="C2" s="3" t="str">
-        <f>VLOOKUP(A2&amp;" - "&amp;B2,name6a,2,FALSE)</f>
+        <f t="shared" ref="C2:C65" si="0">VLOOKUP(A2&amp;" - "&amp;B2,name6a,2,FALSE)</f>
         <v>Yes</v>
       </c>
       <c r="D2" t="s">
@@ -3596,7 +3625,7 @@
         <v>9</v>
       </c>
       <c r="G2" t="s">
-        <v>10</v>
+        <v>239</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
@@ -3607,7 +3636,7 @@
         <v>11</v>
       </c>
       <c r="C3" s="3" t="str">
-        <f>VLOOKUP(A3&amp;" - "&amp;B3,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D3" t="s">
@@ -3631,14 +3660,14 @@
         <v>14</v>
       </c>
       <c r="C4" s="3" t="str">
-        <f>VLOOKUP(A4&amp;" - "&amp;B4,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>
       </c>
       <c r="E4">
-        <v>1921</v>
+        <v>1938</v>
       </c>
       <c r="F4" t="s">
         <v>15</v>
@@ -3655,7 +3684,7 @@
         <v>17</v>
       </c>
       <c r="C5" s="3" t="str">
-        <f>VLOOKUP(A5&amp;" - "&amp;B5,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D5" t="s">
@@ -3679,20 +3708,20 @@
         <v>20</v>
       </c>
       <c r="C6" s="3" t="str">
-        <f>VLOOKUP(A6&amp;" - "&amp;B6,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>To do</v>
       </c>
       <c r="D6" t="s">
         <v>8</v>
       </c>
       <c r="E6">
-        <v>2731</v>
+        <v>2790</v>
       </c>
       <c r="F6" t="s">
         <v>156</v>
       </c>
       <c r="G6" t="s">
-        <v>240</v>
+        <v>231</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
@@ -3703,20 +3732,20 @@
         <v>21</v>
       </c>
       <c r="C7" s="3" t="str">
-        <f>VLOOKUP(A7&amp;" - "&amp;B7,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>To do</v>
       </c>
       <c r="D7" t="s">
         <v>8</v>
       </c>
       <c r="E7">
-        <v>2754</v>
+        <v>2778</v>
       </c>
       <c r="F7" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="G7" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
@@ -3727,20 +3756,20 @@
         <v>22</v>
       </c>
       <c r="C8" s="3" t="str">
-        <f>VLOOKUP(A8&amp;" - "&amp;B8,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>To do</v>
       </c>
       <c r="D8" t="s">
         <v>8</v>
       </c>
       <c r="E8">
-        <v>2757</v>
+        <v>2781</v>
       </c>
       <c r="F8" t="s">
         <v>98</v>
       </c>
       <c r="G8" t="s">
-        <v>237</v>
+        <v>228</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
@@ -3751,20 +3780,20 @@
         <v>23</v>
       </c>
       <c r="C9" s="3" t="str">
-        <f>VLOOKUP(A9&amp;" - "&amp;B9,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>To do</v>
       </c>
       <c r="D9" t="s">
         <v>8</v>
       </c>
       <c r="E9">
-        <v>2762</v>
+        <v>2786</v>
       </c>
       <c r="F9" t="s">
         <v>114</v>
       </c>
       <c r="G9" t="s">
-        <v>236</v>
+        <v>227</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
@@ -3775,20 +3804,20 @@
         <v>24</v>
       </c>
       <c r="C10" s="3" t="str">
-        <f>VLOOKUP(A10&amp;" - "&amp;B10,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>To do</v>
       </c>
       <c r="D10" t="s">
         <v>8</v>
       </c>
       <c r="E10">
-        <v>2755</v>
+        <v>2779</v>
       </c>
       <c r="F10" t="s">
         <v>45</v>
       </c>
       <c r="G10" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
@@ -3799,14 +3828,14 @@
         <v>26</v>
       </c>
       <c r="C11" s="3" t="str">
-        <f>VLOOKUP(A11&amp;" - "&amp;B11,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D11" t="s">
         <v>8</v>
       </c>
       <c r="E11">
-        <v>2522</v>
+        <v>2497</v>
       </c>
       <c r="F11" t="s">
         <v>27</v>
@@ -3823,20 +3852,20 @@
         <v>29</v>
       </c>
       <c r="C12" s="3" t="str">
-        <f>VLOOKUP(A12&amp;" - "&amp;B12,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Note - no need for example</v>
       </c>
       <c r="D12" t="s">
         <v>8</v>
       </c>
       <c r="E12">
-        <v>2553</v>
+        <v>2570</v>
       </c>
       <c r="F12" t="s">
         <v>27</v>
       </c>
       <c r="G12" t="s">
-        <v>234</v>
+        <v>225</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
@@ -3847,20 +3876,20 @@
         <v>30</v>
       </c>
       <c r="C13" s="3" t="str">
-        <f>VLOOKUP(A13&amp;" - "&amp;B13,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Note - no need for example</v>
       </c>
       <c r="D13" t="s">
         <v>8</v>
       </c>
       <c r="E13">
-        <v>2573</v>
+        <v>2590</v>
       </c>
       <c r="F13" t="s">
         <v>27</v>
       </c>
       <c r="G13" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
@@ -3871,20 +3900,20 @@
         <v>31</v>
       </c>
       <c r="C14" s="3" t="str">
-        <f>VLOOKUP(A14&amp;" - "&amp;B14,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Note - no need for example</v>
       </c>
       <c r="D14" t="s">
         <v>8</v>
       </c>
       <c r="E14">
-        <v>2593</v>
+        <v>2610</v>
       </c>
       <c r="F14" t="s">
         <v>27</v>
       </c>
       <c r="G14" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
@@ -3895,20 +3924,20 @@
         <v>32</v>
       </c>
       <c r="C15" s="3" t="str">
-        <f>VLOOKUP(A15&amp;" - "&amp;B15,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Note - no need for example</v>
       </c>
       <c r="D15" t="s">
         <v>8</v>
       </c>
       <c r="E15">
-        <v>2613</v>
+        <v>2630</v>
       </c>
       <c r="F15" t="s">
         <v>27</v>
       </c>
       <c r="G15" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
@@ -3919,20 +3948,20 @@
         <v>33</v>
       </c>
       <c r="C16" s="3" t="str">
-        <f>VLOOKUP(A16&amp;" - "&amp;B16,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Note - no need for example</v>
       </c>
       <c r="D16" t="s">
         <v>8</v>
       </c>
       <c r="E16">
-        <v>2633</v>
+        <v>2650</v>
       </c>
       <c r="F16" t="s">
         <v>27</v>
       </c>
       <c r="G16" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
@@ -3943,20 +3972,20 @@
         <v>34</v>
       </c>
       <c r="C17" s="3" t="str">
-        <f>VLOOKUP(A17&amp;" - "&amp;B17,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Note - no need for example</v>
       </c>
       <c r="D17" t="s">
         <v>8</v>
       </c>
       <c r="E17">
-        <v>2653</v>
+        <v>2670</v>
       </c>
       <c r="F17" t="s">
         <v>27</v>
       </c>
       <c r="G17" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
@@ -3967,20 +3996,20 @@
         <v>35</v>
       </c>
       <c r="C18" s="3" t="str">
-        <f>VLOOKUP(A18&amp;" - "&amp;B18,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Note - no need for example</v>
       </c>
       <c r="D18" t="s">
         <v>8</v>
       </c>
       <c r="E18">
-        <v>2673</v>
+        <v>2690</v>
       </c>
       <c r="F18" t="s">
         <v>27</v>
       </c>
       <c r="G18" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
@@ -3991,14 +4020,14 @@
         <v>37</v>
       </c>
       <c r="C19" s="3" t="str">
-        <f>VLOOKUP(A19&amp;" - "&amp;B19,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D19" t="s">
         <v>8</v>
       </c>
       <c r="E19">
-        <v>2428</v>
+        <v>2445</v>
       </c>
       <c r="F19" t="s">
         <v>12</v>
@@ -4015,20 +4044,20 @@
         <v>39</v>
       </c>
       <c r="C20" s="3" t="str">
-        <f>VLOOKUP(A20&amp;" - "&amp;B20,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>To do</v>
       </c>
       <c r="D20" t="s">
         <v>8</v>
       </c>
       <c r="E20">
-        <v>2373</v>
+        <v>2370</v>
       </c>
       <c r="F20" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
       <c r="G20" t="s">
-        <v>226</v>
+        <v>217</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
@@ -4039,20 +4068,20 @@
         <v>40</v>
       </c>
       <c r="C21" s="3" t="str">
-        <f>VLOOKUP(A21&amp;" - "&amp;B21,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>To do</v>
       </c>
       <c r="D21" t="s">
         <v>8</v>
       </c>
       <c r="E21">
-        <v>2325</v>
+        <v>2392</v>
       </c>
       <c r="F21" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="G21" t="s">
-        <v>224</v>
+        <v>240</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
@@ -4063,14 +4092,14 @@
         <v>41</v>
       </c>
       <c r="C22" s="3" t="str">
-        <f>VLOOKUP(A22&amp;" - "&amp;B22,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D22" t="s">
         <v>8</v>
       </c>
       <c r="E22">
-        <v>2352</v>
+        <v>2369</v>
       </c>
       <c r="F22" t="s">
         <v>42</v>
@@ -4087,20 +4116,20 @@
         <v>44</v>
       </c>
       <c r="C23" s="3" t="str">
-        <f>VLOOKUP(A23&amp;" - "&amp;B23,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D23" t="s">
         <v>8</v>
       </c>
       <c r="E23">
-        <v>2343</v>
+        <v>2360</v>
       </c>
       <c r="F23" t="s">
         <v>45</v>
       </c>
       <c r="G23" t="s">
-        <v>46</v>
+        <v>241</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
@@ -4111,20 +4140,20 @@
         <v>48</v>
       </c>
       <c r="C24" s="3" t="str">
-        <f>VLOOKUP(A24&amp;" - "&amp;B24,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D24" t="s">
         <v>8</v>
       </c>
       <c r="E24">
-        <v>1962</v>
+        <v>1979</v>
       </c>
       <c r="F24" t="s">
-        <v>12</v>
+        <v>242</v>
       </c>
       <c r="G24" t="s">
-        <v>49</v>
+        <v>243</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
@@ -4135,20 +4164,20 @@
         <v>50</v>
       </c>
       <c r="C25" s="3" t="str">
-        <f>VLOOKUP(A25&amp;" - "&amp;B25,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>To do</v>
       </c>
       <c r="D25" t="s">
         <v>8</v>
       </c>
       <c r="E25">
-        <v>1996</v>
+        <v>2013</v>
       </c>
       <c r="F25" t="s">
-        <v>12</v>
+        <v>242</v>
       </c>
       <c r="G25" t="s">
-        <v>223</v>
+        <v>244</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
@@ -4159,20 +4188,20 @@
         <v>51</v>
       </c>
       <c r="C26" s="3" t="str">
-        <f>VLOOKUP(A26&amp;" - "&amp;B26,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>tbd</v>
       </c>
       <c r="D26" t="s">
         <v>8</v>
       </c>
       <c r="E26">
-        <v>2694</v>
+        <v>2711</v>
       </c>
       <c r="F26" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="G26" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
@@ -4183,7 +4212,7 @@
         <v>52</v>
       </c>
       <c r="C27" s="3" t="str">
-        <f>VLOOKUP(A27&amp;" - "&amp;B27,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D27" t="s">
@@ -4207,20 +4236,20 @@
         <v>55</v>
       </c>
       <c r="C28" s="3" t="str">
-        <f>VLOOKUP(A28&amp;" - "&amp;B28,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>To do</v>
       </c>
       <c r="D28" t="s">
         <v>8</v>
       </c>
       <c r="E28">
-        <v>2802</v>
+        <v>2829</v>
       </c>
       <c r="F28" t="s">
         <v>81</v>
       </c>
       <c r="G28" t="s">
-        <v>220</v>
+        <v>245</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
@@ -4231,20 +4260,20 @@
         <v>56</v>
       </c>
       <c r="C29" s="3" t="str">
-        <f>VLOOKUP(A29&amp;" - "&amp;B29,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>To do</v>
       </c>
       <c r="D29" t="s">
         <v>8</v>
       </c>
       <c r="E29">
-        <v>2790</v>
+        <v>2836</v>
       </c>
       <c r="F29" t="s">
         <v>45</v>
       </c>
       <c r="G29" t="s">
-        <v>219</v>
+        <v>246</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.35">
@@ -4255,20 +4284,20 @@
         <v>57</v>
       </c>
       <c r="C30" s="3" t="str">
-        <f>VLOOKUP(A30&amp;" - "&amp;B30,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>To do</v>
       </c>
       <c r="D30" t="s">
         <v>8</v>
       </c>
       <c r="E30">
-        <v>2792</v>
+        <v>2883</v>
       </c>
       <c r="F30" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="G30" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
@@ -4279,20 +4308,20 @@
         <v>58</v>
       </c>
       <c r="C31" s="3" t="str">
-        <f>VLOOKUP(A31&amp;" - "&amp;B31,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>To do</v>
       </c>
       <c r="D31" t="s">
         <v>8</v>
       </c>
       <c r="E31">
-        <v>2791</v>
+        <v>2855</v>
       </c>
       <c r="F31" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="G31" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
@@ -4303,20 +4332,20 @@
         <v>59</v>
       </c>
       <c r="C32" s="3" t="str">
-        <f>VLOOKUP(A32&amp;" - "&amp;B32,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>To do</v>
       </c>
       <c r="D32" t="s">
         <v>8</v>
       </c>
       <c r="E32">
-        <v>2811</v>
+        <v>2842</v>
       </c>
       <c r="F32" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="G32" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
@@ -4327,20 +4356,20 @@
         <v>60</v>
       </c>
       <c r="C33" s="3" t="str">
-        <f>VLOOKUP(A33&amp;" - "&amp;B33,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>To do</v>
       </c>
       <c r="D33" t="s">
         <v>8</v>
       </c>
       <c r="E33">
-        <v>2820</v>
+        <v>2856</v>
       </c>
       <c r="F33" t="s">
         <v>45</v>
       </c>
       <c r="G33" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
@@ -4351,20 +4380,20 @@
         <v>61</v>
       </c>
       <c r="C34" s="3" t="str">
-        <f>VLOOKUP(A34&amp;" - "&amp;B34,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>To do</v>
       </c>
       <c r="D34" t="s">
         <v>8</v>
       </c>
       <c r="E34">
-        <v>2819</v>
+        <v>2870</v>
       </c>
       <c r="F34" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="G34" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
@@ -4375,20 +4404,20 @@
         <v>63</v>
       </c>
       <c r="C35" s="3" t="str">
-        <f>VLOOKUP(A35&amp;" - "&amp;B35,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>To do</v>
       </c>
       <c r="D35" t="s">
         <v>8</v>
       </c>
       <c r="E35">
-        <v>2888</v>
+        <v>2945</v>
       </c>
       <c r="F35" t="s">
         <v>12</v>
       </c>
       <c r="G35" t="s">
-        <v>213</v>
+        <v>247</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
@@ -4399,20 +4428,20 @@
         <v>64</v>
       </c>
       <c r="C36" s="3" t="str">
-        <f>VLOOKUP(A36&amp;" - "&amp;B36,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>To do</v>
       </c>
       <c r="D36" t="s">
         <v>8</v>
       </c>
       <c r="E36">
-        <v>2866</v>
+        <v>2920</v>
       </c>
       <c r="F36" t="s">
         <v>12</v>
       </c>
       <c r="G36" t="s">
-        <v>212</v>
+        <v>248</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
@@ -4423,20 +4452,20 @@
         <v>65</v>
       </c>
       <c r="C37" s="3" t="str">
-        <f>VLOOKUP(A37&amp;" - "&amp;B37,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>To do</v>
       </c>
       <c r="D37" t="s">
         <v>8</v>
       </c>
       <c r="E37">
-        <v>2866</v>
+        <v>2932</v>
       </c>
       <c r="F37" t="s">
         <v>12</v>
       </c>
       <c r="G37" t="s">
-        <v>211</v>
+        <v>249</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
@@ -4447,20 +4476,20 @@
         <v>66</v>
       </c>
       <c r="C38" s="3" t="str">
-        <f>VLOOKUP(A38&amp;" - "&amp;B38,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Mapped</v>
       </c>
       <c r="D38" t="s">
         <v>8</v>
       </c>
       <c r="E38">
-        <v>2899</v>
+        <v>2956</v>
       </c>
       <c r="F38" t="s">
         <v>12</v>
       </c>
       <c r="G38" t="s">
-        <v>210</v>
+        <v>250</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.35">
@@ -4471,20 +4500,20 @@
         <v>67</v>
       </c>
       <c r="C39" s="3" t="str">
-        <f>VLOOKUP(A39&amp;" - "&amp;B39,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D39" t="s">
         <v>8</v>
       </c>
       <c r="E39">
-        <v>1645</v>
+        <v>1644</v>
       </c>
       <c r="F39" t="s">
         <v>68</v>
       </c>
       <c r="G39" t="s">
-        <v>69</v>
+        <v>251</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.35">
@@ -4495,14 +4524,14 @@
         <v>71</v>
       </c>
       <c r="C40" s="3" t="str">
-        <f>VLOOKUP(A40&amp;" - "&amp;B40,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D40" t="s">
         <v>8</v>
       </c>
       <c r="E40">
-        <v>2061</v>
+        <v>2078</v>
       </c>
       <c r="F40" t="s">
         <v>72</v>
@@ -4519,14 +4548,14 @@
         <v>74</v>
       </c>
       <c r="C41" s="3" t="str">
-        <f>VLOOKUP(A41&amp;" - "&amp;B41,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D41" t="s">
         <v>8</v>
       </c>
       <c r="E41">
-        <v>2105</v>
+        <v>2114</v>
       </c>
       <c r="F41" t="s">
         <v>12</v>
@@ -4543,20 +4572,20 @@
         <v>76</v>
       </c>
       <c r="C42" s="3" t="str">
-        <f>VLOOKUP(A42&amp;" - "&amp;B42,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Mapped</v>
       </c>
       <c r="D42" t="s">
         <v>8</v>
       </c>
       <c r="E42">
-        <v>2118</v>
+        <v>2127</v>
       </c>
       <c r="F42" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="G42" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
@@ -4567,14 +4596,14 @@
         <v>77</v>
       </c>
       <c r="C43" s="3" t="str">
-        <f>VLOOKUP(A43&amp;" - "&amp;B43,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D43" t="s">
         <v>8</v>
       </c>
       <c r="E43">
-        <v>2126</v>
+        <v>2136</v>
       </c>
       <c r="F43" t="s">
         <v>78</v>
@@ -4591,14 +4620,14 @@
         <v>80</v>
       </c>
       <c r="C44" s="3" t="str">
-        <f>VLOOKUP(A44&amp;" - "&amp;B44,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D44" t="s">
         <v>8</v>
       </c>
       <c r="E44">
-        <v>2067</v>
+        <v>2124</v>
       </c>
       <c r="F44" t="s">
         <v>81</v>
@@ -4615,20 +4644,20 @@
         <v>83</v>
       </c>
       <c r="C45" s="3" t="str">
-        <f>VLOOKUP(A45&amp;" - "&amp;B45,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Mapped</v>
       </c>
       <c r="D45" t="s">
         <v>8</v>
       </c>
       <c r="E45">
-        <v>2095</v>
+        <v>2132</v>
       </c>
       <c r="F45" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G45" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.35">
@@ -4639,20 +4668,20 @@
         <v>84</v>
       </c>
       <c r="C46" s="3" t="str">
-        <f>VLOOKUP(A46&amp;" - "&amp;B46,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D46" t="s">
         <v>8</v>
       </c>
       <c r="E46">
-        <v>1042</v>
+        <v>1116</v>
       </c>
       <c r="F46" t="s">
         <v>68</v>
       </c>
       <c r="G46" t="s">
-        <v>85</v>
+        <v>252</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.35">
@@ -4663,7 +4692,7 @@
         <v>86</v>
       </c>
       <c r="C47" s="3" t="str">
-        <f>VLOOKUP(A47&amp;" - "&amp;B47,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D47" t="s">
@@ -4687,7 +4716,7 @@
         <v>89</v>
       </c>
       <c r="C48" s="3" t="str">
-        <f>VLOOKUP(A48&amp;" - "&amp;B48,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D48" t="s">
@@ -4711,7 +4740,7 @@
         <v>92</v>
       </c>
       <c r="C49" s="3" t="str">
-        <f>VLOOKUP(A49&amp;" - "&amp;B49,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D49" t="s">
@@ -4724,7 +4753,7 @@
         <v>12</v>
       </c>
       <c r="G49" t="s">
-        <v>93</v>
+        <v>253</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.35">
@@ -4735,14 +4764,14 @@
         <v>94</v>
       </c>
       <c r="C50" s="3" t="str">
-        <f>VLOOKUP(A50&amp;" - "&amp;B50,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D50" t="s">
         <v>8</v>
       </c>
       <c r="E50">
-        <v>1127</v>
+        <v>1131</v>
       </c>
       <c r="F50" t="s">
         <v>95</v>
@@ -4759,14 +4788,14 @@
         <v>97</v>
       </c>
       <c r="C51" s="3" t="str">
-        <f>VLOOKUP(A51&amp;" - "&amp;B51,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D51" t="s">
         <v>8</v>
       </c>
       <c r="E51">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F51" t="s">
         <v>98</v>
@@ -4783,7 +4812,7 @@
         <v>100</v>
       </c>
       <c r="C52" s="3" t="str">
-        <f>VLOOKUP(A52&amp;" - "&amp;B52,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D52" t="s">
@@ -4807,20 +4836,20 @@
         <v>102</v>
       </c>
       <c r="C53" s="3" t="str">
-        <f>VLOOKUP(A53&amp;" - "&amp;B53,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Mapped</v>
       </c>
       <c r="D53" t="s">
         <v>8</v>
       </c>
       <c r="E53">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="F53" t="s">
         <v>114</v>
       </c>
       <c r="G53" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.35">
@@ -4831,7 +4860,7 @@
         <v>103</v>
       </c>
       <c r="C54" s="3" t="str">
-        <f>VLOOKUP(A54&amp;" - "&amp;B54,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D54" t="s">
@@ -4855,7 +4884,7 @@
         <v>106</v>
       </c>
       <c r="C55" s="3" t="str">
-        <f>VLOOKUP(A55&amp;" - "&amp;B55,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D55" t="s">
@@ -4879,20 +4908,20 @@
         <v>109</v>
       </c>
       <c r="C56" s="3" t="str">
-        <f>VLOOKUP(A56&amp;" - "&amp;B56,name6a,2,FALSE)</f>
-        <v>Omit</v>
+        <f t="shared" si="0"/>
+        <v>To do</v>
       </c>
       <c r="D56" t="s">
         <v>8</v>
       </c>
       <c r="E56">
-        <v>1886</v>
+        <v>1892</v>
       </c>
       <c r="F56" t="s">
         <v>12</v>
       </c>
       <c r="G56" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.35">
@@ -4903,7 +4932,7 @@
         <v>110</v>
       </c>
       <c r="C57" s="3" t="str">
-        <f>VLOOKUP(A57&amp;" - "&amp;B57,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D57" t="s">
@@ -4927,14 +4956,14 @@
         <v>113</v>
       </c>
       <c r="C58" s="3" t="str">
-        <f>VLOOKUP(A58&amp;" - "&amp;B58,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D58" t="s">
         <v>8</v>
       </c>
       <c r="E58">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="F58" t="s">
         <v>114</v>
@@ -4951,14 +4980,14 @@
         <v>116</v>
       </c>
       <c r="C59" s="3" t="str">
-        <f>VLOOKUP(A59&amp;" - "&amp;B59,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D59" t="s">
         <v>8</v>
       </c>
       <c r="E59">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="F59" t="s">
         <v>117</v>
@@ -4975,7 +5004,7 @@
         <v>119</v>
       </c>
       <c r="C60" s="3" t="str">
-        <f>VLOOKUP(A60&amp;" - "&amp;B60,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D60" t="s">
@@ -4999,17 +5028,17 @@
         <v>122</v>
       </c>
       <c r="C61" s="3" t="str">
-        <f>VLOOKUP(A61&amp;" - "&amp;B61,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>To do</v>
       </c>
       <c r="D61" t="s">
         <v>8</v>
       </c>
       <c r="E61">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F61" t="s">
-        <v>203</v>
+        <v>254</v>
       </c>
       <c r="G61" t="s">
         <v>202</v>
@@ -5023,14 +5052,14 @@
         <v>123</v>
       </c>
       <c r="C62" s="3" t="str">
-        <f>VLOOKUP(A62&amp;" - "&amp;B62,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>To do</v>
       </c>
       <c r="D62" t="s">
         <v>8</v>
       </c>
       <c r="E62">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F62" t="s">
         <v>201</v>
@@ -5047,7 +5076,7 @@
         <v>124</v>
       </c>
       <c r="C63" s="3" t="str">
-        <f>VLOOKUP(A63&amp;" - "&amp;B63,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D63" t="s">
@@ -5071,14 +5100,14 @@
         <v>127</v>
       </c>
       <c r="C64" s="3" t="str">
-        <f>VLOOKUP(A64&amp;" - "&amp;B64,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D64" t="s">
         <v>8</v>
       </c>
       <c r="E64">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F64" t="s">
         <v>128</v>
@@ -5095,14 +5124,14 @@
         <v>130</v>
       </c>
       <c r="C65" s="3" t="str">
-        <f>VLOOKUP(A65&amp;" - "&amp;B65,name6a,2,FALSE)</f>
+        <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
       <c r="D65" t="s">
         <v>8</v>
       </c>
       <c r="E65">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F65" t="s">
         <v>45</v>
@@ -5119,7 +5148,7 @@
         <v>132</v>
       </c>
       <c r="C66" s="3" t="str">
-        <f>VLOOKUP(A66&amp;" - "&amp;B66,name6a,2,FALSE)</f>
+        <f t="shared" ref="C66:C97" si="1">VLOOKUP(A66&amp;" - "&amp;B66,name6a,2,FALSE)</f>
         <v>Yes</v>
       </c>
       <c r="D66" t="s">
@@ -5143,8 +5172,20 @@
         <v>135</v>
       </c>
       <c r="C67" s="3" t="str">
-        <f>VLOOKUP(A67&amp;" - "&amp;B67,name6a,2,FALSE)</f>
-        <v>Omit</v>
+        <f t="shared" si="1"/>
+        <v>To do</v>
+      </c>
+      <c r="D67" t="s">
+        <v>8</v>
+      </c>
+      <c r="E67">
+        <v>1913</v>
+      </c>
+      <c r="F67" t="s">
+        <v>12</v>
+      </c>
+      <c r="G67" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.35">
@@ -5155,14 +5196,14 @@
         <v>136</v>
       </c>
       <c r="C68" s="3" t="str">
-        <f>VLOOKUP(A68&amp;" - "&amp;B68,name6a,2,FALSE)</f>
-        <v>Omit</v>
+        <f t="shared" si="1"/>
+        <v>To do</v>
       </c>
       <c r="D68" t="s">
         <v>8</v>
       </c>
       <c r="E68">
-        <v>1897</v>
+        <v>1903</v>
       </c>
       <c r="F68" t="s">
         <v>12</v>
@@ -5179,7 +5220,7 @@
         <v>137</v>
       </c>
       <c r="C69" s="3" t="str">
-        <f>VLOOKUP(A69&amp;" - "&amp;B69,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>Mapped</v>
       </c>
     </row>
@@ -5191,7 +5232,7 @@
         <v>138</v>
       </c>
       <c r="C70" s="3" t="str">
-        <f>VLOOKUP(A70&amp;" - "&amp;B70,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>To do</v>
       </c>
     </row>
@@ -5203,7 +5244,7 @@
         <v>139</v>
       </c>
       <c r="C71" s="3" t="str">
-        <f>VLOOKUP(A71&amp;" - "&amp;B71,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
       <c r="D71" t="s">
@@ -5216,7 +5257,7 @@
         <v>12</v>
       </c>
       <c r="G71" t="s">
-        <v>140</v>
+        <v>256</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.35">
@@ -5227,7 +5268,7 @@
         <v>141</v>
       </c>
       <c r="C72" s="3" t="str">
-        <f>VLOOKUP(A72&amp;" - "&amp;B72,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
       <c r="D72" t="s">
@@ -5251,7 +5292,7 @@
         <v>143</v>
       </c>
       <c r="C73" s="3" t="str">
-        <f>VLOOKUP(A73&amp;" - "&amp;B73,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
       <c r="D73" t="s">
@@ -5264,7 +5305,7 @@
         <v>144</v>
       </c>
       <c r="G73" t="s">
-        <v>145</v>
+        <v>257</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.35">
@@ -5275,7 +5316,7 @@
         <v>146</v>
       </c>
       <c r="C74" s="3" t="str">
-        <f>VLOOKUP(A74&amp;" - "&amp;B74,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
       <c r="D74" t="s">
@@ -5288,7 +5329,7 @@
         <v>147</v>
       </c>
       <c r="G74" t="s">
-        <v>148</v>
+        <v>258</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.35">
@@ -5299,7 +5340,7 @@
         <v>149</v>
       </c>
       <c r="C75" s="3" t="str">
-        <f>VLOOKUP(A75&amp;" - "&amp;B75,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
       <c r="D75" t="s">
@@ -5323,7 +5364,7 @@
         <v>151</v>
       </c>
       <c r="C76" s="3" t="str">
-        <f>VLOOKUP(A76&amp;" - "&amp;B76,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
       <c r="D76" t="s">
@@ -5347,14 +5388,14 @@
         <v>153</v>
       </c>
       <c r="C77" s="3" t="str">
-        <f>VLOOKUP(A77&amp;" - "&amp;B77,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>To do</v>
       </c>
       <c r="D77" t="s">
         <v>8</v>
       </c>
       <c r="E77">
-        <v>2911</v>
+        <v>2968</v>
       </c>
       <c r="F77" t="s">
         <v>27</v>
@@ -5371,14 +5412,14 @@
         <v>155</v>
       </c>
       <c r="C78" s="3" t="str">
-        <f>VLOOKUP(A78&amp;" - "&amp;B78,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
       <c r="D78" t="s">
         <v>8</v>
       </c>
       <c r="E78">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F78" t="s">
         <v>156</v>
@@ -5395,7 +5436,7 @@
         <v>158</v>
       </c>
       <c r="C79" s="3" t="str">
-        <f>VLOOKUP(A79&amp;" - "&amp;B79,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
       <c r="D79" t="s">
@@ -5419,7 +5460,7 @@
         <v>161</v>
       </c>
       <c r="C80" s="3" t="str">
-        <f>VLOOKUP(A80&amp;" - "&amp;B80,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
       <c r="D80" t="s">
@@ -5443,7 +5484,7 @@
         <v>163</v>
       </c>
       <c r="C81" s="3" t="str">
-        <f>VLOOKUP(A81&amp;" - "&amp;B81,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
       <c r="D81" t="s">
@@ -5467,14 +5508,14 @@
         <v>166</v>
       </c>
       <c r="C82" s="3" t="str">
-        <f>VLOOKUP(A82&amp;" - "&amp;B82,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
       <c r="D82" t="s">
         <v>8</v>
       </c>
       <c r="E82">
-        <v>1862</v>
+        <v>1861</v>
       </c>
       <c r="F82" t="s">
         <v>12</v>
@@ -5491,14 +5532,14 @@
         <v>168</v>
       </c>
       <c r="C83" s="3" t="str">
-        <f>VLOOKUP(A83&amp;" - "&amp;B83,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>Later</v>
       </c>
       <c r="D83" t="s">
         <v>8</v>
       </c>
       <c r="E83">
-        <v>1908</v>
+        <v>1925</v>
       </c>
       <c r="F83" t="s">
         <v>12</v>
@@ -5515,20 +5556,20 @@
         <v>170</v>
       </c>
       <c r="C84" s="3" t="str">
-        <f>VLOOKUP(A84&amp;" - "&amp;B84,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>Yes</v>
       </c>
       <c r="D84" t="s">
         <v>8</v>
       </c>
       <c r="E84">
-        <v>1456</v>
+        <v>1454</v>
       </c>
       <c r="F84" t="s">
         <v>9</v>
       </c>
       <c r="G84" t="s">
-        <v>171</v>
+        <v>259</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.35">
@@ -5539,14 +5580,14 @@
         <v>173</v>
       </c>
       <c r="C85" s="3" t="str">
-        <f>VLOOKUP(A85&amp;" - "&amp;B85,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>Mapped</v>
       </c>
       <c r="D85" t="s">
         <v>8</v>
       </c>
       <c r="E85">
-        <v>2241</v>
+        <v>2258</v>
       </c>
       <c r="F85" t="s">
         <v>12</v>
@@ -5563,14 +5604,14 @@
         <v>174</v>
       </c>
       <c r="C86" s="3" t="str">
-        <f>VLOOKUP(A86&amp;" - "&amp;B86,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>Mapped</v>
       </c>
       <c r="D86" t="s">
         <v>8</v>
       </c>
       <c r="E86">
-        <v>2205</v>
+        <v>2222</v>
       </c>
       <c r="F86" t="s">
         <v>12</v>
@@ -5587,14 +5628,14 @@
         <v>175</v>
       </c>
       <c r="C87" s="3" t="str">
-        <f>VLOOKUP(A87&amp;" - "&amp;B87,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>Mapped</v>
       </c>
       <c r="D87" t="s">
         <v>8</v>
       </c>
       <c r="E87">
-        <v>2193</v>
+        <v>2210</v>
       </c>
       <c r="F87" t="s">
         <v>12</v>
@@ -5611,14 +5652,14 @@
         <v>176</v>
       </c>
       <c r="C88" s="3" t="str">
-        <f>VLOOKUP(A88&amp;" - "&amp;B88,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>Mapped</v>
       </c>
       <c r="D88" t="s">
         <v>8</v>
       </c>
       <c r="E88">
-        <v>2217</v>
+        <v>2234</v>
       </c>
       <c r="F88" t="s">
         <v>12</v>
@@ -5635,14 +5676,14 @@
         <v>177</v>
       </c>
       <c r="C89" s="3" t="str">
-        <f>VLOOKUP(A89&amp;" - "&amp;B89,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>Mapped</v>
       </c>
       <c r="D89" t="s">
         <v>8</v>
       </c>
       <c r="E89">
-        <v>2253</v>
+        <v>2270</v>
       </c>
       <c r="F89" t="s">
         <v>12</v>
@@ -5659,14 +5700,14 @@
         <v>178</v>
       </c>
       <c r="C90" s="3" t="str">
-        <f>VLOOKUP(A90&amp;" - "&amp;B90,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>Mapped</v>
       </c>
       <c r="D90" t="s">
         <v>8</v>
       </c>
       <c r="E90">
-        <v>2229</v>
+        <v>2246</v>
       </c>
       <c r="F90" t="s">
         <v>12</v>
@@ -5683,14 +5724,14 @@
         <v>179</v>
       </c>
       <c r="C91" s="3" t="str">
-        <f>VLOOKUP(A91&amp;" - "&amp;B91,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>Mapped</v>
       </c>
       <c r="D91" t="s">
         <v>8</v>
       </c>
       <c r="E91">
-        <v>2178</v>
+        <v>2195</v>
       </c>
       <c r="F91" t="s">
         <v>12</v>
@@ -5707,14 +5748,14 @@
         <v>181</v>
       </c>
       <c r="C92" s="3" t="str">
-        <f>VLOOKUP(A92&amp;" - "&amp;B92,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>Mapped</v>
       </c>
       <c r="D92" t="s">
         <v>8</v>
       </c>
       <c r="E92">
-        <v>2289</v>
+        <v>2306</v>
       </c>
       <c r="F92" t="s">
         <v>12</v>
@@ -5731,7 +5772,7 @@
         <v>182</v>
       </c>
       <c r="C93" s="3" t="str">
-        <f>VLOOKUP(A93&amp;" - "&amp;B93,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>Mapped</v>
       </c>
     </row>
@@ -5743,7 +5784,7 @@
         <v>183</v>
       </c>
       <c r="C94" s="3" t="str">
-        <f>VLOOKUP(A94&amp;" - "&amp;B94,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>Mapped</v>
       </c>
     </row>
@@ -5755,7 +5796,7 @@
         <v>184</v>
       </c>
       <c r="C95" s="3" t="str">
-        <f>VLOOKUP(A95&amp;" - "&amp;B95,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>Mapped</v>
       </c>
     </row>
@@ -5767,14 +5808,14 @@
         <v>185</v>
       </c>
       <c r="C96" s="3" t="str">
-        <f>VLOOKUP(A96&amp;" - "&amp;B96,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>Mapped</v>
       </c>
       <c r="D96" t="s">
         <v>8</v>
       </c>
       <c r="E96">
-        <v>2277</v>
+        <v>2294</v>
       </c>
       <c r="F96" t="s">
         <v>12</v>
@@ -5791,14 +5832,14 @@
         <v>186</v>
       </c>
       <c r="C97" s="3" t="str">
-        <f>VLOOKUP(A97&amp;" - "&amp;B97,name6a,2,FALSE)</f>
+        <f t="shared" si="1"/>
         <v>Mapped</v>
       </c>
       <c r="D97" t="s">
         <v>8</v>
       </c>
       <c r="E97">
-        <v>2265</v>
+        <v>2282</v>
       </c>
       <c r="F97" t="s">
         <v>12</v>

</xml_diff>